<commit_message>
Fix BP forecast calibration with training-only model selection
</commit_message>
<xml_diff>
--- a/results/三路径预测_BP_最新/五SSP三路径需水预测_最新.xlsx
+++ b/results/三路径预测_BP_最新/五SSP三路径需水预测_最新.xlsx
@@ -19,13 +19,16 @@
     <sheet name="历史回测" sheetId="11" r:id="rId13"/>
     <sheet name="误差指标" sheetId="12" r:id="rId14"/>
     <sheet name="参数与口径" sheetId="13" r:id="rId15"/>
+    <sheet name="主模型_效率保持" sheetId="14" r:id="rId16"/>
+    <sheet name="主模型_历史趋势" sheetId="15" r:id="rId17"/>
+    <sheet name="主模型_规划约束" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="369" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="756" uniqueCount="105">
   <si>
     <t>年份</t>
   </si>
@@ -322,6 +325,24 @@
   </si>
   <si>
     <t>分行业重构量是估计参考，未替换训练驱动；面积为播种代理；工业火电口径未完全统一</t>
+  </si>
+  <si>
+    <t>发展变化_剔除基期衔接差</t>
+  </si>
+  <si>
+    <t>基期衔接差_含校准与效率</t>
+  </si>
+  <si>
+    <t>基期衔接差</t>
+  </si>
+  <si>
+    <t>3-1-1正则BP、12成员；随机小初值直接局部训练，无PSO；正则与last/none/median3校准在训练期内联合选择</t>
+  </si>
+  <si>
+    <t>近期均值效率下2023反事实预测165.055297276；总衔接差0.055297276，其中预测校准衔接差0.000000000，效率差0.055297276；均不计入发展效应</t>
+  </si>
+  <si>
+    <t>政策净变化=发展变化+基期衔接差−历史节水−额外政策节水；均为模型条件差异，不是政策因果效应</t>
   </si>
 </sst>
 </file>
@@ -370,10 +391,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="19.42578125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -423,13 +444,13 @@
         <v>2025</v>
       </c>
       <c r="B4" s="0">
-        <v>165.30180939577485</v>
+        <v>165.30180939577482</v>
       </c>
       <c r="C4" s="0">
         <v>163.97336291396618</v>
       </c>
       <c r="D4" s="0">
-        <v>163.80656719074852</v>
+        <v>163.8065671907485</v>
       </c>
     </row>
     <row r="5">
@@ -443,7 +464,7 @@
         <v>163.55132054552689</v>
       </c>
       <c r="D5" s="0">
-        <v>163.31537043441051</v>
+        <v>163.31537043441048</v>
       </c>
     </row>
     <row r="6">
@@ -454,10 +475,10 @@
         <v>165.66473162170803</v>
       </c>
       <c r="C6" s="0">
-        <v>163.21259564728871</v>
+        <v>163.21259564728874</v>
       </c>
       <c r="D6" s="0">
-        <v>162.91468122506888</v>
+        <v>162.91468122506885</v>
       </c>
     </row>
     <row r="7">
@@ -465,13 +486,13 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>165.92452240193279</v>
+        <v>165.92452240193282</v>
       </c>
       <c r="C7" s="0">
-        <v>162.94645336639951</v>
+        <v>162.94645336639954</v>
       </c>
       <c r="D7" s="0">
-        <v>162.59229900031778</v>
+        <v>162.59229900031775</v>
       </c>
     </row>
     <row r="8">
@@ -479,13 +500,13 @@
         <v>2029</v>
       </c>
       <c r="B8" s="0">
-        <v>166.23235054936822</v>
+        <v>166.23235054936825</v>
       </c>
       <c r="C8" s="0">
-        <v>162.74433075594322</v>
+        <v>162.74433075594325</v>
       </c>
       <c r="D8" s="0">
-        <v>162.33840659579766</v>
+        <v>162.33840659579769</v>
       </c>
     </row>
     <row r="9">
@@ -499,7 +520,7 @@
         <v>162.59936305964357</v>
       </c>
       <c r="D9" s="0">
-        <v>162.14507925618148</v>
+        <v>162.1450792561815</v>
       </c>
     </row>
   </sheetData>
@@ -511,20 +532,20 @@
   <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="14.85546875" customWidth="true"/>
-    <col min="3" max="3" width="16.42578125" customWidth="true"/>
-    <col min="4" max="4" width="27.140625" customWidth="true"/>
-    <col min="5" max="5" width="32.5703125" customWidth="true"/>
-    <col min="6" max="6" width="32.5703125" customWidth="true"/>
-    <col min="7" max="7" width="32.5703125" customWidth="true"/>
-    <col min="8" max="8" width="31.7109375" customWidth="true"/>
-    <col min="9" max="9" width="27" customWidth="true"/>
-    <col min="10" max="10" width="34.85546875" customWidth="true"/>
-    <col min="11" max="11" width="33.85546875" customWidth="true"/>
-    <col min="12" max="12" width="26.85546875" customWidth="true"/>
-    <col min="13" max="13" width="33.28515625" customWidth="true"/>
-    <col min="14" max="14" width="24.140625" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="7.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="16.7109375" customWidth="true"/>
+    <col min="5" max="5" width="17.7109375" customWidth="true"/>
+    <col min="6" max="6" width="17.7109375" customWidth="true"/>
+    <col min="7" max="7" width="17.7109375" customWidth="true"/>
+    <col min="8" max="8" width="15.7109375" customWidth="true"/>
+    <col min="9" max="9" width="14.7109375" customWidth="true"/>
+    <col min="10" max="10" width="18.7109375" customWidth="true"/>
+    <col min="11" max="11" width="17.7109375" customWidth="true"/>
+    <col min="12" max="12" width="17.7109375" customWidth="true"/>
+    <col min="13" max="13" width="19.7109375" customWidth="true"/>
+    <col min="14" max="14" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1196,9 +1217,9 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="12.5703125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="6.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
     <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
@@ -1224,10 +1245,10 @@
         <v>166.90000000000001</v>
       </c>
       <c r="C2" s="0">
-        <v>169.84222793612653</v>
+        <v>170.54050281151692</v>
       </c>
       <c r="D2" s="0">
-        <v>169.84222793612653</v>
+        <v>170.54050281151692</v>
       </c>
     </row>
     <row r="3">
@@ -1238,10 +1259,10 @@
         <v>164.5</v>
       </c>
       <c r="C3" s="0">
-        <v>165.44547853849704</v>
+        <v>166.14375341388737</v>
       </c>
       <c r="D3" s="0">
-        <v>161.73000921482887</v>
+        <v>163.32646567999592</v>
       </c>
     </row>
     <row r="4">
@@ -1252,10 +1273,10 @@
         <v>194.30000000000001</v>
       </c>
       <c r="C4" s="0">
-        <v>165.44306151477943</v>
+        <v>166.14133639016976</v>
       </c>
       <c r="D4" s="0">
-        <v>164.51439156863458</v>
+        <v>164.35392612979754</v>
       </c>
     </row>
     <row r="5">
@@ -1266,10 +1287,10 @@
         <v>165</v>
       </c>
       <c r="C5" s="0">
-        <v>165.31376203821966</v>
+        <v>166.01203691361002</v>
       </c>
       <c r="D5" s="0">
-        <v>193.85139612124465</v>
+        <v>174.12252338801076</v>
       </c>
     </row>
   </sheetData>
@@ -1281,10 +1302,10 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="true"/>
-    <col min="2" max="2" width="13.140625" customWidth="true"/>
-    <col min="3" max="3" width="10.7109375" customWidth="true"/>
-    <col min="4" max="4" width="10.7109375" customWidth="true"/>
+    <col min="1" max="1" width="5.7109375" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
     <col min="5" max="5" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
@@ -1310,16 +1331,16 @@
         <v>68</v>
       </c>
       <c r="B2" s="0">
-        <v>4.3448826228715962</v>
+        <v>4.5715525065171096</v>
       </c>
       <c r="C2" s="0">
-        <v>8.2646017495159541</v>
+        <v>8.613739187211138</v>
       </c>
       <c r="D2" s="0">
-        <v>14.511822596174079</v>
+        <v>14.229280911314676</v>
       </c>
       <c r="E2" s="0">
-        <v>210.59299506282858</v>
+        <v>202.47243525310421</v>
       </c>
     </row>
     <row r="3">
@@ -1327,16 +1348,16 @@
         <v>69</v>
       </c>
       <c r="B3" s="0">
-        <v>9.065537256341905</v>
+        <v>5.9589329586260522</v>
       </c>
       <c r="C3" s="0">
-        <v>16.087305818476935</v>
+        <v>10.970658597433555</v>
       </c>
       <c r="D3" s="0">
-        <v>20.832157125161416</v>
+        <v>15.768784169406629</v>
       </c>
       <c r="E3" s="0">
-        <v>433.97877048741361</v>
+        <v>248.6545541813291</v>
       </c>
     </row>
   </sheetData>
@@ -1348,8 +1369,8 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" customWidth="true"/>
-    <col min="2" max="2" width="116.85546875" customWidth="true"/>
+    <col min="1" max="1" width="9.7109375" customWidth="true"/>
+    <col min="2" max="2" width="91.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1365,7 +1386,7 @@
         <v>75</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3">
@@ -1418,10 +1439,10 @@
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>11</v>
+        <v>101</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10">
@@ -1429,7 +1450,7 @@
         <v>82</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11">
@@ -1454,6 +1475,597 @@
       </c>
       <c r="B13" s="0" t="s">
         <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>2023</v>
+      </c>
+      <c r="B2" s="0">
+        <v>165</v>
+      </c>
+      <c r="C2" s="0">
+        <v>165</v>
+      </c>
+      <c r="D2" s="0">
+        <v>165</v>
+      </c>
+      <c r="E2" s="0">
+        <v>165</v>
+      </c>
+      <c r="F2" s="0">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="0">
+        <v>165.18863526492498</v>
+      </c>
+      <c r="C3" s="0">
+        <v>165.17908275339116</v>
+      </c>
+      <c r="D3" s="0">
+        <v>165.17701487907493</v>
+      </c>
+      <c r="E3" s="0">
+        <v>165.1895952774822</v>
+      </c>
+      <c r="F3" s="0">
+        <v>165.19379656327158</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="0">
+        <v>165.30180939577482</v>
+      </c>
+      <c r="C4" s="0">
+        <v>165.2711738744573</v>
+      </c>
+      <c r="D4" s="0">
+        <v>165.35738468088491</v>
+      </c>
+      <c r="E4" s="0">
+        <v>165.31187985390261</v>
+      </c>
+      <c r="F4" s="0">
+        <v>165.21639502021847</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="0">
+        <v>165.45586062647601</v>
+      </c>
+      <c r="C5" s="0">
+        <v>165.39175668478586</v>
+      </c>
+      <c r="D5" s="0">
+        <v>165.55205244119807</v>
+      </c>
+      <c r="E5" s="0">
+        <v>165.48313209048629</v>
+      </c>
+      <c r="F5" s="0">
+        <v>165.28897196681351</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2027</v>
+      </c>
+      <c r="B6" s="0">
+        <v>165.66473162170803</v>
+      </c>
+      <c r="C6" s="0">
+        <v>165.55366021191779</v>
+      </c>
+      <c r="D6" s="0">
+        <v>165.77368046029872</v>
+      </c>
+      <c r="E6" s="0">
+        <v>165.71745574966292</v>
+      </c>
+      <c r="F6" s="0">
+        <v>165.42417374238485</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>2028</v>
+      </c>
+      <c r="B7" s="0">
+        <v>165.92452240193282</v>
+      </c>
+      <c r="C7" s="0">
+        <v>165.75165500037545</v>
+      </c>
+      <c r="D7" s="0">
+        <v>166.01647565182864</v>
+      </c>
+      <c r="E7" s="0">
+        <v>166.01099013827528</v>
+      </c>
+      <c r="F7" s="0">
+        <v>165.61699065494943</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>2029</v>
+      </c>
+      <c r="B8" s="0">
+        <v>166.23235054936825</v>
+      </c>
+      <c r="C8" s="0">
+        <v>165.98140207955001</v>
+      </c>
+      <c r="D8" s="0">
+        <v>166.2752704578138</v>
+      </c>
+      <c r="E8" s="0">
+        <v>166.36088331665101</v>
+      </c>
+      <c r="F8" s="0">
+        <v>165.86358790002359</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>2030</v>
+      </c>
+      <c r="B9" s="0">
+        <v>166.58603768167302</v>
+      </c>
+      <c r="C9" s="0">
+        <v>166.23919280151537</v>
+      </c>
+      <c r="D9" s="0">
+        <v>166.54533035125226</v>
+      </c>
+      <c r="E9" s="0">
+        <v>166.76496394097839</v>
+      </c>
+      <c r="F9" s="0">
+        <v>166.16095993962062</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>2023</v>
+      </c>
+      <c r="B2" s="0">
+        <v>165</v>
+      </c>
+      <c r="C2" s="0">
+        <v>165</v>
+      </c>
+      <c r="D2" s="0">
+        <v>165</v>
+      </c>
+      <c r="E2" s="0">
+        <v>165</v>
+      </c>
+      <c r="F2" s="0">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="0">
+        <v>164.4748707566232</v>
+      </c>
+      <c r="C3" s="0">
+        <v>164.56953805219825</v>
+      </c>
+      <c r="D3" s="0">
+        <v>164.67302725600658</v>
+      </c>
+      <c r="E3" s="0">
+        <v>164.57953360994256</v>
+      </c>
+      <c r="F3" s="0">
+        <v>164.47896102783025</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="0">
+        <v>163.97336291396618</v>
+      </c>
+      <c r="C4" s="0">
+        <v>164.13567579262497</v>
+      </c>
+      <c r="D4" s="0">
+        <v>164.41462707096798</v>
+      </c>
+      <c r="E4" s="0">
+        <v>164.17326296256701</v>
+      </c>
+      <c r="F4" s="0">
+        <v>163.89090552699315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="0">
+        <v>163.55132054552689</v>
+      </c>
+      <c r="C5" s="0">
+        <v>163.75690974914644</v>
+      </c>
+      <c r="D5" s="0">
+        <v>164.18191529280378</v>
+      </c>
+      <c r="E5" s="0">
+        <v>163.8388305998279</v>
+      </c>
+      <c r="F5" s="0">
+        <v>163.39477302566306</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2027</v>
+      </c>
+      <c r="B6" s="0">
+        <v>163.21259564728874</v>
+      </c>
+      <c r="C6" s="0">
+        <v>163.43991055875333</v>
+      </c>
+      <c r="D6" s="0">
+        <v>163.98491070706658</v>
+      </c>
+      <c r="E6" s="0">
+        <v>163.58262820418608</v>
+      </c>
+      <c r="F6" s="0">
+        <v>162.99175619689834</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>2028</v>
+      </c>
+      <c r="B7" s="0">
+        <v>162.94645336639954</v>
+      </c>
+      <c r="C7" s="0">
+        <v>163.17580300969129</v>
+      </c>
+      <c r="D7" s="0">
+        <v>163.81713336301104</v>
+      </c>
+      <c r="E7" s="0">
+        <v>163.39575223633111</v>
+      </c>
+      <c r="F7" s="0">
+        <v>162.66880106233478</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>2029</v>
+      </c>
+      <c r="B8" s="0">
+        <v>162.74433075594325</v>
+      </c>
+      <c r="C8" s="0">
+        <v>162.9573087336141</v>
+      </c>
+      <c r="D8" s="0">
+        <v>163.673153193015</v>
+      </c>
+      <c r="E8" s="0">
+        <v>163.27120556907315</v>
+      </c>
+      <c r="F8" s="0">
+        <v>162.41535206017434</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>2030</v>
+      </c>
+      <c r="B9" s="0">
+        <v>162.59936305964357</v>
+      </c>
+      <c r="C9" s="0">
+        <v>162.77836104508094</v>
+      </c>
+      <c r="D9" s="0">
+        <v>163.54829125244339</v>
+      </c>
+      <c r="E9" s="0">
+        <v>163.20348132848176</v>
+      </c>
+      <c r="F9" s="0">
+        <v>162.22283681275971</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0">
+        <v>2023</v>
+      </c>
+      <c r="B2" s="0">
+        <v>165</v>
+      </c>
+      <c r="C2" s="0">
+        <v>165</v>
+      </c>
+      <c r="D2" s="0">
+        <v>165</v>
+      </c>
+      <c r="E2" s="0">
+        <v>165</v>
+      </c>
+      <c r="F2" s="0">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0">
+        <v>2024</v>
+      </c>
+      <c r="B3" s="0">
+        <v>164.38619132866143</v>
+      </c>
+      <c r="C3" s="0">
+        <v>164.46117903195341</v>
+      </c>
+      <c r="D3" s="0">
+        <v>164.54470676967648</v>
+      </c>
+      <c r="E3" s="0">
+        <v>164.47111208956099</v>
+      </c>
+      <c r="F3" s="0">
+        <v>164.3902603462378</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="0">
+        <v>163.8065671907485</v>
+      </c>
+      <c r="C4" s="0">
+        <v>163.93019403217457</v>
+      </c>
+      <c r="D4" s="0">
+        <v>164.16796436844359</v>
+      </c>
+      <c r="E4" s="0">
+        <v>163.96729971165348</v>
+      </c>
+      <c r="F4" s="0">
+        <v>163.72499472037973</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0">
+        <v>2026</v>
+      </c>
+      <c r="B5" s="0">
+        <v>163.31537043441048</v>
+      </c>
+      <c r="C5" s="0">
+        <v>163.46416615192814</v>
+      </c>
+      <c r="D5" s="0">
+        <v>163.82594933505655</v>
+      </c>
+      <c r="E5" s="0">
+        <v>163.54448971731844</v>
+      </c>
+      <c r="F5" s="0">
+        <v>163.16139254018776</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0">
+        <v>2027</v>
+      </c>
+      <c r="B6" s="0">
+        <v>162.91468122506885</v>
+      </c>
+      <c r="C6" s="0">
+        <v>163.06813799635407</v>
+      </c>
+      <c r="D6" s="0">
+        <v>163.52743712330894</v>
+      </c>
+      <c r="E6" s="0">
+        <v>163.20712392957537</v>
+      </c>
+      <c r="F6" s="0">
+        <v>162.698715825823</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0">
+        <v>2028</v>
+      </c>
+      <c r="B7" s="0">
+        <v>162.59229900031775</v>
+      </c>
+      <c r="C7" s="0">
+        <v>162.73191661247611</v>
+      </c>
+      <c r="D7" s="0">
+        <v>163.26502966281927</v>
+      </c>
+      <c r="E7" s="0">
+        <v>162.9446861805086</v>
+      </c>
+      <c r="F7" s="0">
+        <v>162.32230473874094</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0">
+        <v>2029</v>
+      </c>
+      <c r="B8" s="0">
+        <v>162.33840659579769</v>
+      </c>
+      <c r="C8" s="0">
+        <v>162.44709821255762</v>
+      </c>
+      <c r="D8" s="0">
+        <v>163.03254975774743</v>
+      </c>
+      <c r="E8" s="0">
+        <v>162.74878569972665</v>
+      </c>
+      <c r="F8" s="0">
+        <v>162.02023833242632</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0">
+        <v>2030</v>
+      </c>
+      <c r="B9" s="0">
+        <v>162.1450792561815</v>
+      </c>
+      <c r="C9" s="0">
+        <v>162.20666765288874</v>
+      </c>
+      <c r="D9" s="0">
+        <v>162.82472202834637</v>
+      </c>
+      <c r="E9" s="0">
+        <v>162.61272343277821</v>
+      </c>
+      <c r="F9" s="0">
+        <v>161.78280304265581</v>
       </c>
     </row>
   </sheetData>
@@ -1465,10 +2077,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="19.42578125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1504,7 +2116,7 @@
         <v>2024</v>
       </c>
       <c r="B3" s="0">
-        <v>165.17908275339119</v>
+        <v>165.17908275339116</v>
       </c>
       <c r="C3" s="0">
         <v>164.56953805219825</v>
@@ -1524,7 +2136,7 @@
         <v>164.13567579262497</v>
       </c>
       <c r="D4" s="0">
-        <v>163.93019403217454</v>
+        <v>163.93019403217457</v>
       </c>
     </row>
     <row r="5">
@@ -1532,13 +2144,13 @@
         <v>2026</v>
       </c>
       <c r="B5" s="0">
-        <v>165.39175668478583</v>
+        <v>165.39175668478586</v>
       </c>
       <c r="C5" s="0">
-        <v>163.75690974914642</v>
+        <v>163.75690974914644</v>
       </c>
       <c r="D5" s="0">
-        <v>163.46416615192811</v>
+        <v>163.46416615192814</v>
       </c>
     </row>
     <row r="6">
@@ -1546,13 +2158,13 @@
         <v>2027</v>
       </c>
       <c r="B6" s="0">
-        <v>165.55366021191776</v>
+        <v>165.55366021191779</v>
       </c>
       <c r="C6" s="0">
-        <v>163.43991055875335</v>
+        <v>163.43991055875333</v>
       </c>
       <c r="D6" s="0">
-        <v>163.06813799635404</v>
+        <v>163.06813799635407</v>
       </c>
     </row>
     <row r="7">
@@ -1560,13 +2172,13 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>165.75165500037542</v>
+        <v>165.75165500037545</v>
       </c>
       <c r="C7" s="0">
-        <v>163.17580300969121</v>
+        <v>163.17580300969129</v>
       </c>
       <c r="D7" s="0">
-        <v>162.73191661247608</v>
+        <v>162.73191661247611</v>
       </c>
     </row>
     <row r="8">
@@ -1574,13 +2186,13 @@
         <v>2029</v>
       </c>
       <c r="B8" s="0">
-        <v>165.98140207954998</v>
+        <v>165.98140207955001</v>
       </c>
       <c r="C8" s="0">
-        <v>162.95730873361413</v>
+        <v>162.9573087336141</v>
       </c>
       <c r="D8" s="0">
-        <v>162.44709821255765</v>
+        <v>162.44709821255762</v>
       </c>
     </row>
     <row r="9">
@@ -1588,13 +2200,13 @@
         <v>2030</v>
       </c>
       <c r="B9" s="0">
-        <v>166.2391928015154</v>
+        <v>166.23919280151537</v>
       </c>
       <c r="C9" s="0">
         <v>162.77836104508094</v>
       </c>
       <c r="D9" s="0">
-        <v>162.20666765288877</v>
+        <v>162.20666765288874</v>
       </c>
     </row>
   </sheetData>
@@ -1606,10 +2218,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="19.42578125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1648,10 +2260,10 @@
         <v>165.17701487907493</v>
       </c>
       <c r="C3" s="0">
-        <v>164.67302725600655</v>
+        <v>164.67302725600658</v>
       </c>
       <c r="D3" s="0">
-        <v>164.54470676967651</v>
+        <v>164.54470676967648</v>
       </c>
     </row>
     <row r="4">
@@ -1659,13 +2271,13 @@
         <v>2025</v>
       </c>
       <c r="B4" s="0">
-        <v>165.35738468088493</v>
+        <v>165.35738468088491</v>
       </c>
       <c r="C4" s="0">
         <v>164.41462707096798</v>
       </c>
       <c r="D4" s="0">
-        <v>164.16796436844356</v>
+        <v>164.16796436844359</v>
       </c>
     </row>
     <row r="5">
@@ -1673,13 +2285,13 @@
         <v>2026</v>
       </c>
       <c r="B5" s="0">
-        <v>165.55205244119804</v>
+        <v>165.55205244119807</v>
       </c>
       <c r="C5" s="0">
-        <v>164.18191529280375</v>
+        <v>164.18191529280378</v>
       </c>
       <c r="D5" s="0">
-        <v>163.82594933505652</v>
+        <v>163.82594933505655</v>
       </c>
     </row>
     <row r="6">
@@ -1687,13 +2299,13 @@
         <v>2027</v>
       </c>
       <c r="B6" s="0">
-        <v>165.77368046029869</v>
+        <v>165.77368046029872</v>
       </c>
       <c r="C6" s="0">
-        <v>163.98491070706655</v>
+        <v>163.98491070706658</v>
       </c>
       <c r="D6" s="0">
-        <v>163.52743712330891</v>
+        <v>163.52743712330894</v>
       </c>
     </row>
     <row r="7">
@@ -1701,13 +2313,13 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>166.01647565182861</v>
+        <v>166.01647565182864</v>
       </c>
       <c r="C7" s="0">
-        <v>163.81713336301107</v>
+        <v>163.81713336301104</v>
       </c>
       <c r="D7" s="0">
-        <v>163.2650296628193</v>
+        <v>163.26502966281927</v>
       </c>
     </row>
     <row r="8">
@@ -1718,10 +2330,10 @@
         <v>166.2752704578138</v>
       </c>
       <c r="C8" s="0">
-        <v>163.67315319301497</v>
+        <v>163.673153193015</v>
       </c>
       <c r="D8" s="0">
-        <v>163.03254975774746</v>
+        <v>163.03254975774743</v>
       </c>
     </row>
     <row r="9">
@@ -1729,13 +2341,13 @@
         <v>2030</v>
       </c>
       <c r="B9" s="0">
-        <v>166.54533035125223</v>
+        <v>166.54533035125226</v>
       </c>
       <c r="C9" s="0">
         <v>163.54829125244339</v>
       </c>
       <c r="D9" s="0">
-        <v>162.8247220283464</v>
+        <v>162.82472202834637</v>
       </c>
     </row>
   </sheetData>
@@ -1747,10 +2359,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="19.42578125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1786,13 +2398,13 @@
         <v>2024</v>
       </c>
       <c r="B3" s="0">
-        <v>165.18959527748223</v>
+        <v>165.1895952774822</v>
       </c>
       <c r="C3" s="0">
-        <v>164.57953360994259</v>
+        <v>164.57953360994256</v>
       </c>
       <c r="D3" s="0">
-        <v>164.47111208956096</v>
+        <v>164.47111208956099</v>
       </c>
     </row>
     <row r="4">
@@ -1803,7 +2415,7 @@
         <v>165.31187985390261</v>
       </c>
       <c r="C4" s="0">
-        <v>164.17326296256704</v>
+        <v>164.17326296256701</v>
       </c>
       <c r="D4" s="0">
         <v>163.96729971165348</v>
@@ -1814,13 +2426,13 @@
         <v>2026</v>
       </c>
       <c r="B5" s="0">
-        <v>165.48313209048638</v>
+        <v>165.48313209048629</v>
       </c>
       <c r="C5" s="0">
-        <v>163.83883059982793</v>
+        <v>163.8388305998279</v>
       </c>
       <c r="D5" s="0">
-        <v>163.54448971731847</v>
+        <v>163.54448971731844</v>
       </c>
     </row>
     <row r="6">
@@ -1831,10 +2443,10 @@
         <v>165.71745574966292</v>
       </c>
       <c r="C6" s="0">
-        <v>163.58262820418611</v>
+        <v>163.58262820418608</v>
       </c>
       <c r="D6" s="0">
-        <v>163.20712392957535</v>
+        <v>163.20712392957537</v>
       </c>
     </row>
     <row r="7">
@@ -1842,10 +2454,10 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>166.01099013827525</v>
+        <v>166.01099013827528</v>
       </c>
       <c r="C7" s="0">
-        <v>163.39575223633108</v>
+        <v>163.39575223633111</v>
       </c>
       <c r="D7" s="0">
         <v>162.9446861805086</v>
@@ -1856,13 +2468,13 @@
         <v>2029</v>
       </c>
       <c r="B8" s="0">
-        <v>166.36088331665098</v>
+        <v>166.36088331665101</v>
       </c>
       <c r="C8" s="0">
-        <v>163.27120556907312</v>
+        <v>163.27120556907315</v>
       </c>
       <c r="D8" s="0">
-        <v>162.74878569972668</v>
+        <v>162.74878569972665</v>
       </c>
     </row>
     <row r="9">
@@ -1870,13 +2482,13 @@
         <v>2030</v>
       </c>
       <c r="B9" s="0">
-        <v>166.76496394097842</v>
+        <v>166.76496394097839</v>
       </c>
       <c r="C9" s="0">
         <v>163.20348132848176</v>
       </c>
       <c r="D9" s="0">
-        <v>162.61272343277824</v>
+        <v>162.61272343277821</v>
       </c>
     </row>
   </sheetData>
@@ -1888,10 +2500,10 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="19.42578125" customWidth="true"/>
-    <col min="3" max="3" width="14.85546875" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1930,10 +2542,10 @@
         <v>165.19379656327158</v>
       </c>
       <c r="C3" s="0">
-        <v>164.47896102783022</v>
+        <v>164.47896102783025</v>
       </c>
       <c r="D3" s="0">
-        <v>164.39026034623782</v>
+        <v>164.3902603462378</v>
       </c>
     </row>
     <row r="4">
@@ -1941,13 +2553,13 @@
         <v>2025</v>
       </c>
       <c r="B4" s="0">
-        <v>165.21639502021844</v>
+        <v>165.21639502021847</v>
       </c>
       <c r="C4" s="0">
         <v>163.89090552699315</v>
       </c>
       <c r="D4" s="0">
-        <v>163.72499472037975</v>
+        <v>163.72499472037973</v>
       </c>
     </row>
     <row r="5">
@@ -1958,7 +2570,7 @@
         <v>165.28897196681351</v>
       </c>
       <c r="C5" s="0">
-        <v>163.39477302566308</v>
+        <v>163.39477302566306</v>
       </c>
       <c r="D5" s="0">
         <v>163.16139254018776</v>
@@ -1969,7 +2581,7 @@
         <v>2027</v>
       </c>
       <c r="B6" s="0">
-        <v>165.42417374238482</v>
+        <v>165.42417374238485</v>
       </c>
       <c r="C6" s="0">
         <v>162.99175619689834</v>
@@ -1983,13 +2595,13 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>165.6169906549494</v>
+        <v>165.61699065494943</v>
       </c>
       <c r="C7" s="0">
-        <v>162.66880106233475</v>
+        <v>162.66880106233478</v>
       </c>
       <c r="D7" s="0">
-        <v>162.32230473874097</v>
+        <v>162.32230473874094</v>
       </c>
     </row>
     <row r="8">
@@ -1997,13 +2609,13 @@
         <v>2029</v>
       </c>
       <c r="B8" s="0">
-        <v>165.86358790002362</v>
+        <v>165.86358790002359</v>
       </c>
       <c r="C8" s="0">
-        <v>162.41535206017431</v>
+        <v>162.41535206017434</v>
       </c>
       <c r="D8" s="0">
-        <v>162.02023833242629</v>
+        <v>162.02023833242632</v>
       </c>
     </row>
     <row r="9">
@@ -2014,7 +2626,7 @@
         <v>166.16095993962062</v>
       </c>
       <c r="C9" s="0">
-        <v>162.22283681275974</v>
+        <v>162.22283681275971</v>
       </c>
       <c r="D9" s="0">
         <v>161.78280304265581</v>
@@ -2029,20 +2641,20 @@
   <dimension ref="A1:N36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="5.7109375" customWidth="true"/>
-    <col min="3" max="3" width="19.42578125" customWidth="true"/>
-    <col min="4" max="4" width="14.85546875" customWidth="true"/>
-    <col min="5" max="5" width="14.85546875" customWidth="true"/>
-    <col min="6" max="6" width="29.5703125" customWidth="true"/>
-    <col min="7" max="7" width="14.85546875" customWidth="true"/>
-    <col min="8" max="8" width="14.85546875" customWidth="true"/>
-    <col min="9" max="9" width="14.85546875" customWidth="true"/>
+    <col min="1" max="1" width="5.28515625" customWidth="true"/>
+    <col min="2" max="2" width="5.140625" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="13.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13.7109375" customWidth="true"/>
+    <col min="8" max="8" width="12.7109375" customWidth="true"/>
+    <col min="9" max="9" width="13.7109375" customWidth="true"/>
     <col min="10" max="10" width="12.7109375" customWidth="true"/>
-    <col min="11" max="11" width="21.140625" customWidth="true"/>
-    <col min="12" max="12" width="19.42578125" customWidth="true"/>
-    <col min="13" max="13" width="18.85546875" customWidth="true"/>
-    <col min="14" max="14" width="17.140625" customWidth="true"/>
+    <col min="11" max="11" width="13.42578125" customWidth="true"/>
+    <col min="12" max="12" width="11.7109375" customWidth="true"/>
+    <col min="13" max="13" width="11.7109375" customWidth="true"/>
+    <col min="14" max="14" width="8.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2062,10 +2674,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>11</v>
+        <v>100</v>
       </c>
       <c r="H1" s="0" t="s">
         <v>12</v>
@@ -2106,10 +2718,10 @@
         <v>164.38619132866143</v>
       </c>
       <c r="F2" s="0">
-        <v>0.13333798908308836</v>
+        <v>0.13333798908311678</v>
       </c>
       <c r="G2" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H2" s="0">
         <v>0.71376450830177873</v>
@@ -2124,7 +2736,7 @@
         <v>-0.61380867133857464</v>
       </c>
       <c r="L2" s="0">
-        <v>6.0181193805429443</v>
+        <v>6.0181193805416617</v>
       </c>
       <c r="M2" s="0"/>
       <c r="N2" s="0"/>
@@ -2137,31 +2749,31 @@
         <v>2025</v>
       </c>
       <c r="C3" s="0">
-        <v>165.30180939577485</v>
+        <v>165.30180939577482</v>
       </c>
       <c r="D3" s="0">
         <v>163.97336291396618</v>
       </c>
       <c r="E3" s="0">
-        <v>163.80656719074852</v>
+        <v>163.8065671907485</v>
       </c>
       <c r="F3" s="0">
         <v>0.24651211993295874</v>
       </c>
       <c r="G3" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H3" s="0">
-        <v>1.328446481808669</v>
+        <v>1.3284464818086406</v>
       </c>
       <c r="I3" s="0">
-        <v>0.16679572321766045</v>
+        <v>0.16679572321768887</v>
       </c>
       <c r="J3" s="0">
         <v>1.4952422050263294</v>
       </c>
       <c r="K3" s="0">
-        <v>-1.1934328092514761</v>
+        <v>-1.1934328092515045</v>
       </c>
       <c r="L3" s="0">
         <v>6.0655930646857215</v>
@@ -2183,28 +2795,28 @@
         <v>163.55132054552689</v>
       </c>
       <c r="E4" s="0">
-        <v>163.31537043441051</v>
+        <v>163.31537043441048</v>
       </c>
       <c r="F4" s="0">
-        <v>0.40056335063411552</v>
+        <v>0.40056335063414394</v>
       </c>
       <c r="G4" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H4" s="0">
         <v>1.9045400809491184</v>
       </c>
       <c r="I4" s="0">
-        <v>0.23595011111638087</v>
+        <v>0.23595011111640929</v>
       </c>
       <c r="J4" s="0">
-        <v>2.1404901920654993</v>
+        <v>2.1404901920655277</v>
       </c>
       <c r="K4" s="0">
-        <v>-1.6846295655894892</v>
+        <v>-1.6846295655895176</v>
       </c>
       <c r="L4" s="0">
-        <v>5.3436995388544073</v>
+        <v>5.3436995388540991</v>
       </c>
       <c r="M4" s="0"/>
       <c r="N4" s="0"/>
@@ -2220,31 +2832,31 @@
         <v>165.66473162170803</v>
       </c>
       <c r="D5" s="0">
-        <v>163.21259564728871</v>
+        <v>163.21259564728874</v>
       </c>
       <c r="E5" s="0">
-        <v>162.91468122506888</v>
+        <v>162.91468122506885</v>
       </c>
       <c r="F5" s="0">
-        <v>0.60943434586613421</v>
+        <v>0.60943434586616263</v>
       </c>
       <c r="G5" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H5" s="0">
-        <v>2.4521359744193205</v>
+        <v>2.4521359744192921</v>
       </c>
       <c r="I5" s="0">
-        <v>0.29791442221983289</v>
+        <v>0.29791442221988973</v>
       </c>
       <c r="J5" s="0">
-        <v>2.7500503966391534</v>
+        <v>2.7500503966391818</v>
       </c>
       <c r="K5" s="0">
-        <v>-2.0853187749311246</v>
+        <v>-2.085318774931153</v>
       </c>
       <c r="L5" s="0">
-        <v>4.5124637547802697</v>
+        <v>4.5124637547801054</v>
       </c>
       <c r="M5" s="0"/>
       <c r="N5" s="0"/>
@@ -2257,34 +2869,34 @@
         <v>2028</v>
       </c>
       <c r="C6" s="0">
-        <v>165.92452240193279</v>
+        <v>165.92452240193282</v>
       </c>
       <c r="D6" s="0">
-        <v>162.94645336639951</v>
+        <v>162.94645336639954</v>
       </c>
       <c r="E6" s="0">
-        <v>162.59229900031778</v>
+        <v>162.59229900031775</v>
       </c>
       <c r="F6" s="0">
-        <v>0.86922512609089608</v>
+        <v>0.86922512609095293</v>
       </c>
       <c r="G6" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H6" s="0">
         <v>2.9780690355332808</v>
       </c>
       <c r="I6" s="0">
-        <v>0.35415436608172968</v>
+        <v>0.35415436608178652</v>
       </c>
       <c r="J6" s="0">
-        <v>3.3322234016150105</v>
+        <v>3.3322234016150674</v>
       </c>
       <c r="K6" s="0">
-        <v>-2.4077009996822198</v>
+        <v>-2.4077009996822483</v>
       </c>
       <c r="L6" s="0">
-        <v>3.8335562348511258</v>
+        <v>3.8335562348509402</v>
       </c>
       <c r="M6" s="0"/>
       <c r="N6" s="0"/>
@@ -2297,19 +2909,19 @@
         <v>2029</v>
       </c>
       <c r="C7" s="0">
-        <v>166.23235054936822</v>
+        <v>166.23235054936825</v>
       </c>
       <c r="D7" s="0">
-        <v>162.74433075594322</v>
+        <v>162.74433075594325</v>
       </c>
       <c r="E7" s="0">
-        <v>162.33840659579766</v>
+        <v>162.33840659579769</v>
       </c>
       <c r="F7" s="0">
-        <v>1.1770532735263259</v>
+        <v>1.1770532735263828</v>
       </c>
       <c r="G7" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H7" s="0">
         <v>3.4880197934249964</v>
@@ -2321,10 +2933,10 @@
         <v>3.893943953570556</v>
       </c>
       <c r="K7" s="0">
-        <v>-2.6615934042023355</v>
+        <v>-2.6615934042023071</v>
       </c>
       <c r="L7" s="0">
-        <v>3.3082138601124789</v>
+        <v>3.308213860112319</v>
       </c>
       <c r="M7" s="0"/>
       <c r="N7" s="0"/>
@@ -2343,28 +2955,28 @@
         <v>162.59936305964357</v>
       </c>
       <c r="E8" s="0">
-        <v>162.14507925618148</v>
+        <v>162.1450792561815</v>
       </c>
       <c r="F8" s="0">
-        <v>1.5307404058311249</v>
+        <v>1.5307404058311533</v>
       </c>
       <c r="G8" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H8" s="0">
         <v>3.9866746220294544</v>
       </c>
       <c r="I8" s="0">
-        <v>0.45428380346208996</v>
+        <v>0.45428380346206154</v>
       </c>
       <c r="J8" s="0">
-        <v>4.4409584254915444</v>
+        <v>4.440958425491516</v>
       </c>
       <c r="K8" s="0">
-        <v>-2.8549207438185249</v>
+        <v>-2.8549207438184965</v>
       </c>
       <c r="L8" s="0">
-        <v>2.9011832499974406</v>
+        <v>2.9011832499973682</v>
       </c>
       <c r="M8" s="0">
         <v>173.25866293314667</v>
@@ -2381,7 +2993,7 @@
         <v>2024</v>
       </c>
       <c r="C9" s="0">
-        <v>165.17908275339119</v>
+        <v>165.17908275339116</v>
       </c>
       <c r="D9" s="0">
         <v>164.56953805219825</v>
@@ -2393,22 +3005,22 @@
         <v>0.12378547754929059</v>
       </c>
       <c r="G9" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H9" s="0">
-        <v>0.60954470119293092</v>
+        <v>0.60954470119290249</v>
       </c>
       <c r="I9" s="0">
         <v>0.10835902024484767</v>
       </c>
       <c r="J9" s="0">
-        <v>0.71790372143777859</v>
+        <v>0.71790372143775016</v>
       </c>
       <c r="K9" s="0">
         <v>-0.53882096804659341</v>
       </c>
       <c r="L9" s="0">
-        <v>5.7995795278320426</v>
+        <v>5.7995795278318125</v>
       </c>
       <c r="M9" s="0"/>
       <c r="N9" s="0"/>
@@ -2427,28 +3039,28 @@
         <v>164.13567579262497</v>
       </c>
       <c r="E10" s="0">
-        <v>163.93019403217454</v>
+        <v>163.93019403217457</v>
       </c>
       <c r="F10" s="0">
-        <v>0.21587659861540942</v>
+        <v>0.21587659861543784</v>
       </c>
       <c r="G10" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H10" s="0">
         <v>1.1354980818323384</v>
       </c>
       <c r="I10" s="0">
-        <v>0.2054817604504251</v>
+        <v>0.20548176045039668</v>
       </c>
       <c r="J10" s="0">
-        <v>1.3409798422827635</v>
+        <v>1.340979842282735</v>
       </c>
       <c r="K10" s="0">
-        <v>-1.0698059678254594</v>
+        <v>-1.069805967825431</v>
       </c>
       <c r="L10" s="0">
-        <v>6.2117888223343698</v>
+        <v>6.2117888223334203</v>
       </c>
       <c r="M10" s="0"/>
       <c r="N10" s="0"/>
@@ -2461,19 +3073,19 @@
         <v>2026</v>
       </c>
       <c r="C11" s="0">
-        <v>165.39175668478583</v>
+        <v>165.39175668478586</v>
       </c>
       <c r="D11" s="0">
-        <v>163.75690974914642</v>
+        <v>163.75690974914644</v>
       </c>
       <c r="E11" s="0">
-        <v>163.46416615192811</v>
+        <v>163.46416615192814</v>
       </c>
       <c r="F11" s="0">
-        <v>0.33645940894393789</v>
+        <v>0.33645940894399473</v>
       </c>
       <c r="G11" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H11" s="0">
         <v>1.6348469356394162</v>
@@ -2485,10 +3097,10 @@
         <v>1.927590532857721</v>
       </c>
       <c r="K11" s="0">
-        <v>-1.5358338480718885</v>
+        <v>-1.5358338480718601</v>
       </c>
       <c r="L11" s="0">
-        <v>5.7290433306886754</v>
+        <v>5.7290433306877073</v>
       </c>
       <c r="M11" s="0"/>
       <c r="N11" s="0"/>
@@ -2501,34 +3113,34 @@
         <v>2027</v>
       </c>
       <c r="C12" s="0">
-        <v>165.55366021191776</v>
+        <v>165.55366021191779</v>
       </c>
       <c r="D12" s="0">
-        <v>163.43991055875335</v>
+        <v>163.43991055875333</v>
       </c>
       <c r="E12" s="0">
-        <v>163.06813799635404</v>
+        <v>163.06813799635407</v>
       </c>
       <c r="F12" s="0">
-        <v>0.49836293607586413</v>
+        <v>0.49836293607592097</v>
       </c>
       <c r="G12" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H12" s="0">
-        <v>2.1137496531644047</v>
+        <v>2.1137496531644615</v>
       </c>
       <c r="I12" s="0">
-        <v>0.37177256239931467</v>
+        <v>0.37177256239925782</v>
       </c>
       <c r="J12" s="0">
         <v>2.4855222155637193</v>
       </c>
       <c r="K12" s="0">
-        <v>-1.9318620036459606</v>
+        <v>-1.9318620036459322</v>
       </c>
       <c r="L12" s="0">
-        <v>4.9873737303477093</v>
+        <v>4.9873737303471399</v>
       </c>
       <c r="M12" s="0"/>
       <c r="N12" s="0"/>
@@ -2541,34 +3153,34 @@
         <v>2028</v>
       </c>
       <c r="C13" s="0">
-        <v>165.75165500037542</v>
+        <v>165.75165500037545</v>
       </c>
       <c r="D13" s="0">
-        <v>163.17580300969121</v>
+        <v>163.17580300969129</v>
       </c>
       <c r="E13" s="0">
-        <v>162.73191661247608</v>
+        <v>162.73191661247611</v>
       </c>
       <c r="F13" s="0">
-        <v>0.69635772453352729</v>
+        <v>0.69635772453358413</v>
       </c>
       <c r="G13" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H13" s="0">
-        <v>2.5758519906842139</v>
+        <v>2.575851990684157</v>
       </c>
       <c r="I13" s="0">
-        <v>0.44388639721512391</v>
+        <v>0.44388639721518075</v>
       </c>
       <c r="J13" s="0">
         <v>3.0197383878993378</v>
       </c>
       <c r="K13" s="0">
-        <v>-2.2680833875239159</v>
+        <v>-2.2680833875238875</v>
       </c>
       <c r="L13" s="0">
-        <v>4.3364757530652591</v>
+        <v>4.3364757530649047</v>
       </c>
       <c r="M13" s="0"/>
       <c r="N13" s="0"/>
@@ -2581,34 +3193,34 @@
         <v>2029</v>
       </c>
       <c r="C14" s="0">
-        <v>165.98140207954998</v>
+        <v>165.98140207955001</v>
       </c>
       <c r="D14" s="0">
-        <v>162.95730873361413</v>
+        <v>162.9573087336141</v>
       </c>
       <c r="E14" s="0">
-        <v>162.44709821255765</v>
+        <v>162.44709821255762</v>
       </c>
       <c r="F14" s="0">
-        <v>0.92610480370808546</v>
+        <v>0.9261048037081423</v>
       </c>
       <c r="G14" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H14" s="0">
-        <v>3.024093345935853</v>
+        <v>3.0240933459359098</v>
       </c>
       <c r="I14" s="0">
         <v>0.51021052105647868</v>
       </c>
       <c r="J14" s="0">
-        <v>3.5343038669923317</v>
+        <v>3.5343038669923885</v>
       </c>
       <c r="K14" s="0">
-        <v>-2.5529017874423516</v>
+        <v>-2.5529017874423801</v>
       </c>
       <c r="L14" s="0">
-        <v>3.8163109108614108</v>
+        <v>3.8163109108612381</v>
       </c>
       <c r="M14" s="0"/>
       <c r="N14" s="0"/>
@@ -2621,31 +3233,31 @@
         <v>2030</v>
       </c>
       <c r="C15" s="0">
-        <v>166.2391928015154</v>
+        <v>166.23919280151537</v>
       </c>
       <c r="D15" s="0">
         <v>162.77836104508094</v>
       </c>
       <c r="E15" s="0">
-        <v>162.20666765288877</v>
+        <v>162.20666765288874</v>
       </c>
       <c r="F15" s="0">
         <v>1.1838955256735062</v>
       </c>
       <c r="G15" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H15" s="0">
-        <v>3.4608317564344588</v>
+        <v>3.4608317564344304</v>
       </c>
       <c r="I15" s="0">
-        <v>0.57169339219217363</v>
+        <v>0.57169339219220205</v>
       </c>
       <c r="J15" s="0">
         <v>4.0325251486266325</v>
       </c>
       <c r="K15" s="0">
-        <v>-2.7933323471112317</v>
+        <v>-2.7933323471112601</v>
       </c>
       <c r="L15" s="0">
         <v>3.4061494964537262</v>
@@ -2668,31 +3280,31 @@
         <v>165.17701487907493</v>
       </c>
       <c r="D16" s="0">
-        <v>164.67302725600655</v>
+        <v>164.67302725600658</v>
       </c>
       <c r="E16" s="0">
-        <v>164.54470676967651</v>
+        <v>164.54470676967648</v>
       </c>
       <c r="F16" s="0">
-        <v>0.12171760323303715</v>
+        <v>0.12171760323306557</v>
       </c>
       <c r="G16" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H16" s="0">
-        <v>0.50398762306838307</v>
+        <v>0.50398762306835465</v>
       </c>
       <c r="I16" s="0">
-        <v>0.12832048633003978</v>
+        <v>0.12832048633009663</v>
       </c>
       <c r="J16" s="0">
-        <v>0.63230810939842286</v>
+        <v>0.63230810939845128</v>
       </c>
       <c r="K16" s="0">
-        <v>-0.45529323032349112</v>
+        <v>-0.45529323032351954</v>
       </c>
       <c r="L16" s="0">
-        <v>5.1948780833929442</v>
+        <v>5.1948780833919646</v>
       </c>
       <c r="M16" s="0"/>
       <c r="N16" s="0"/>
@@ -2705,34 +3317,34 @@
         <v>2025</v>
       </c>
       <c r="C17" s="0">
-        <v>165.35738468088493</v>
+        <v>165.35738468088491</v>
       </c>
       <c r="D17" s="0">
         <v>164.41462707096798</v>
       </c>
       <c r="E17" s="0">
-        <v>164.16796436844356</v>
+        <v>164.16796436844359</v>
       </c>
       <c r="F17" s="0">
         <v>0.30208740504303933</v>
       </c>
       <c r="G17" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H17" s="0">
-        <v>0.94275760991695279</v>
+        <v>0.94275760991692437</v>
       </c>
       <c r="I17" s="0">
-        <v>0.24666270252441791</v>
+        <v>0.24666270252438949</v>
       </c>
       <c r="J17" s="0">
-        <v>1.1894203124413707</v>
+        <v>1.1894203124413139</v>
       </c>
       <c r="K17" s="0">
-        <v>-0.83203563155643678</v>
+        <v>-0.83203563155640836</v>
       </c>
       <c r="L17" s="0">
-        <v>3.9373383086657001</v>
+        <v>3.9373383086655118</v>
       </c>
       <c r="M17" s="0"/>
       <c r="N17" s="0"/>
@@ -2745,19 +3357,19 @@
         <v>2026</v>
       </c>
       <c r="C18" s="0">
-        <v>165.55205244119804</v>
+        <v>165.55205244119807</v>
       </c>
       <c r="D18" s="0">
-        <v>164.18191529280375</v>
+        <v>164.18191529280378</v>
       </c>
       <c r="E18" s="0">
-        <v>163.82594933505652</v>
+        <v>163.82594933505655</v>
       </c>
       <c r="F18" s="0">
-        <v>0.49675516535614861</v>
+        <v>0.49675516535620545</v>
       </c>
       <c r="G18" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H18" s="0">
         <v>1.3701371483942921</v>
@@ -2769,10 +3381,10 @@
         <v>1.7261031061415224</v>
       </c>
       <c r="K18" s="0">
-        <v>-1.1740506649434792</v>
+        <v>-1.1740506649434508</v>
       </c>
       <c r="L18" s="0">
-        <v>3.4747562310781266</v>
+        <v>3.4747562310777287</v>
       </c>
       <c r="M18" s="0"/>
       <c r="N18" s="0"/>
@@ -2785,19 +3397,19 @@
         <v>2027</v>
       </c>
       <c r="C19" s="0">
-        <v>165.77368046029869</v>
+        <v>165.77368046029872</v>
       </c>
       <c r="D19" s="0">
-        <v>163.98491070706655</v>
+        <v>163.98491070706658</v>
       </c>
       <c r="E19" s="0">
-        <v>163.52743712330891</v>
+        <v>163.52743712330894</v>
       </c>
       <c r="F19" s="0">
-        <v>0.71838318445679761</v>
+        <v>0.71838318445685445</v>
       </c>
       <c r="G19" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H19" s="0">
         <v>1.7887697532321454</v>
@@ -2809,10 +3421,10 @@
         <v>2.2462433369897781</v>
       </c>
       <c r="K19" s="0">
-        <v>-1.4725628766910859</v>
+        <v>-1.4725628766910575</v>
       </c>
       <c r="L19" s="0">
-        <v>3.126803891837008</v>
+        <v>3.1268038918367607</v>
       </c>
       <c r="M19" s="0"/>
       <c r="N19" s="0"/>
@@ -2825,34 +3437,34 @@
         <v>2028</v>
       </c>
       <c r="C20" s="0">
-        <v>166.01647565182861</v>
+        <v>166.01647565182864</v>
       </c>
       <c r="D20" s="0">
-        <v>163.81713336301107</v>
+        <v>163.81713336301104</v>
       </c>
       <c r="E20" s="0">
-        <v>163.2650296628193</v>
+        <v>163.26502966281927</v>
       </c>
       <c r="F20" s="0">
-        <v>0.9611783759867194</v>
+        <v>0.96117837598677625</v>
       </c>
       <c r="G20" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H20" s="0">
-        <v>2.1993422888175473</v>
+        <v>2.1993422888176042</v>
       </c>
       <c r="I20" s="0">
         <v>0.5521037001917648</v>
       </c>
       <c r="J20" s="0">
-        <v>2.7514459890093121</v>
+        <v>2.751445989009369</v>
       </c>
       <c r="K20" s="0">
-        <v>-1.7349703371806982</v>
+        <v>-1.7349703371807266</v>
       </c>
       <c r="L20" s="0">
-        <v>2.8625758316553398</v>
+        <v>2.8625758316552297</v>
       </c>
       <c r="M20" s="0"/>
       <c r="N20" s="0"/>
@@ -2868,31 +3480,31 @@
         <v>166.2752704578138</v>
       </c>
       <c r="D21" s="0">
-        <v>163.67315319301497</v>
+        <v>163.673153193015</v>
       </c>
       <c r="E21" s="0">
-        <v>163.03254975774746</v>
+        <v>163.03254975774743</v>
       </c>
       <c r="F21" s="0">
-        <v>1.2199731819719091</v>
+        <v>1.2199731819719375</v>
       </c>
       <c r="G21" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H21" s="0">
-        <v>2.6021172647988351</v>
+        <v>2.6021172647988067</v>
       </c>
       <c r="I21" s="0">
-        <v>0.64060343526750785</v>
+        <v>0.64060343526756469</v>
       </c>
       <c r="J21" s="0">
-        <v>3.2427207000663429</v>
+        <v>3.2427207000663714</v>
       </c>
       <c r="K21" s="0">
-        <v>-1.9674502422525393</v>
+        <v>-1.9674502422525677</v>
       </c>
       <c r="L21" s="0">
-        <v>2.6580262156459513</v>
+        <v>2.6580262156459127</v>
       </c>
       <c r="M21" s="0"/>
       <c r="N21" s="0"/>
@@ -2905,34 +3517,34 @@
         <v>2030</v>
       </c>
       <c r="C22" s="0">
-        <v>166.54533035125223</v>
+        <v>166.54533035125226</v>
       </c>
       <c r="D22" s="0">
         <v>163.54829125244339</v>
       </c>
       <c r="E22" s="0">
-        <v>162.8247220283464</v>
+        <v>162.82472202834637</v>
       </c>
       <c r="F22" s="0">
-        <v>1.4900330754103379</v>
+        <v>1.4900330754103948</v>
       </c>
       <c r="G22" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H22" s="0">
-        <v>2.9970390988088411</v>
+        <v>2.9970390988088695</v>
       </c>
       <c r="I22" s="0">
-        <v>0.72356922409699109</v>
+        <v>0.72356922409701951</v>
       </c>
       <c r="J22" s="0">
-        <v>3.7206083229058322</v>
+        <v>3.7206083229058891</v>
       </c>
       <c r="K22" s="0">
-        <v>-2.1752779716535997</v>
+        <v>-2.1752779716536281</v>
       </c>
       <c r="L22" s="0">
-        <v>2.4969971367120287</v>
+        <v>2.4969971367119719</v>
       </c>
       <c r="M22" s="0">
         <v>173.25866293314667</v>
@@ -2949,34 +3561,34 @@
         <v>2024</v>
       </c>
       <c r="C23" s="0">
-        <v>165.18959527748223</v>
+        <v>165.1895952774822</v>
       </c>
       <c r="D23" s="0">
-        <v>164.57953360994259</v>
+        <v>164.57953360994256</v>
       </c>
       <c r="E23" s="0">
-        <v>164.47111208956096</v>
+        <v>164.47111208956099</v>
       </c>
       <c r="F23" s="0">
         <v>0.13429800164033168</v>
       </c>
       <c r="G23" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H23" s="0">
         <v>0.61006166753963953</v>
       </c>
       <c r="I23" s="0">
-        <v>0.10842152038162567</v>
+        <v>0.10842152038156883</v>
       </c>
       <c r="J23" s="0">
-        <v>0.7184831879212652</v>
+        <v>0.71848318792120835</v>
       </c>
       <c r="K23" s="0">
-        <v>-0.52888791043903893</v>
+        <v>-0.52888791043901051</v>
       </c>
       <c r="L23" s="0">
-        <v>5.3499171927029927</v>
+        <v>5.3499171927025699</v>
       </c>
       <c r="M23" s="0"/>
       <c r="N23" s="0"/>
@@ -2992,22 +3604,22 @@
         <v>165.31187985390261</v>
       </c>
       <c r="D24" s="0">
-        <v>164.17326296256704</v>
+        <v>164.17326296256701</v>
       </c>
       <c r="E24" s="0">
         <v>163.96729971165348</v>
       </c>
       <c r="F24" s="0">
-        <v>0.2565825780607156</v>
+        <v>0.25658257806074403</v>
       </c>
       <c r="G24" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H24" s="0">
-        <v>1.1386168913355732</v>
+        <v>1.1386168913356016</v>
       </c>
       <c r="I24" s="0">
-        <v>0.20596325091355538</v>
+        <v>0.20596325091352696</v>
       </c>
       <c r="J24" s="0">
         <v>1.3445801422491286</v>
@@ -3016,7 +3628,7 @@
         <v>-1.0327002883465184</v>
       </c>
       <c r="L24" s="0">
-        <v>5.2403407605132024</v>
+        <v>5.2403407605126224</v>
       </c>
       <c r="M24" s="0"/>
       <c r="N24" s="0"/>
@@ -3029,34 +3641,34 @@
         <v>2026</v>
       </c>
       <c r="C25" s="0">
-        <v>165.48313209048638</v>
+        <v>165.48313209048629</v>
       </c>
       <c r="D25" s="0">
-        <v>163.83883059982793</v>
+        <v>163.8388305998279</v>
       </c>
       <c r="E25" s="0">
-        <v>163.54448971731847</v>
+        <v>163.54448971731844</v>
       </c>
       <c r="F25" s="0">
-        <v>0.42783481464448414</v>
+        <v>0.4278348146444273</v>
       </c>
       <c r="G25" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H25" s="0">
-        <v>1.6443014906584494</v>
+        <v>1.6443014906583926</v>
       </c>
       <c r="I25" s="0">
         <v>0.29434088250945933</v>
       </c>
       <c r="J25" s="0">
-        <v>1.9386423731679088</v>
+        <v>1.9386423731678519</v>
       </c>
       <c r="K25" s="0">
-        <v>-1.45551028268153</v>
+        <v>-1.4555102826815585</v>
       </c>
       <c r="L25" s="0">
-        <v>4.531287092142918</v>
+        <v>4.531287092143387</v>
       </c>
       <c r="M25" s="0"/>
       <c r="N25" s="0"/>
@@ -3072,31 +3684,31 @@
         <v>165.71745574966292</v>
       </c>
       <c r="D26" s="0">
-        <v>163.58262820418611</v>
+        <v>163.58262820418608</v>
       </c>
       <c r="E26" s="0">
-        <v>163.20712392957535</v>
+        <v>163.20712392957537</v>
       </c>
       <c r="F26" s="0">
-        <v>0.66215847382102311</v>
+        <v>0.66215847382105153</v>
       </c>
       <c r="G26" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H26" s="0">
-        <v>2.13482754547681</v>
+        <v>2.1348275454768384</v>
       </c>
       <c r="I26" s="0">
-        <v>0.37550427461076197</v>
+        <v>0.37550427461070512</v>
       </c>
       <c r="J26" s="0">
-        <v>2.5103318200875719</v>
+        <v>2.5103318200875435</v>
       </c>
       <c r="K26" s="0">
-        <v>-1.7928760704246542</v>
+        <v>-1.7928760704246258</v>
       </c>
       <c r="L26" s="0">
-        <v>3.7911344781281127</v>
+        <v>3.791134478127907</v>
       </c>
       <c r="M26" s="0"/>
       <c r="N26" s="0"/>
@@ -3109,34 +3721,34 @@
         <v>2028</v>
       </c>
       <c r="C27" s="0">
-        <v>166.01099013827525</v>
+        <v>166.01099013827528</v>
       </c>
       <c r="D27" s="0">
-        <v>163.39575223633108</v>
+        <v>163.39575223633111</v>
       </c>
       <c r="E27" s="0">
         <v>162.9446861805086</v>
       </c>
       <c r="F27" s="0">
-        <v>0.95569286243335227</v>
+        <v>0.95569286243340912</v>
       </c>
       <c r="G27" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H27" s="0">
         <v>2.6152379019441696</v>
       </c>
       <c r="I27" s="0">
-        <v>0.45106605582247994</v>
+        <v>0.45106605582250836</v>
       </c>
       <c r="J27" s="0">
-        <v>3.0663039577666495</v>
+        <v>3.066303957766678</v>
       </c>
       <c r="K27" s="0">
         <v>-2.0553138194914027</v>
       </c>
       <c r="L27" s="0">
-        <v>3.208461712227642</v>
+        <v>3.2084617122274808</v>
       </c>
       <c r="M27" s="0"/>
       <c r="N27" s="0"/>
@@ -3149,34 +3761,34 @@
         <v>2029</v>
       </c>
       <c r="C28" s="0">
-        <v>166.36088331665098</v>
+        <v>166.36088331665101</v>
       </c>
       <c r="D28" s="0">
-        <v>163.27120556907312</v>
+        <v>163.27120556907315</v>
       </c>
       <c r="E28" s="0">
-        <v>162.74878569972668</v>
+        <v>162.74878569972665</v>
       </c>
       <c r="F28" s="0">
-        <v>1.3055860408090894</v>
+        <v>1.3055860408091462</v>
       </c>
       <c r="G28" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H28" s="0">
         <v>3.0896777475778663</v>
       </c>
       <c r="I28" s="0">
-        <v>0.52241986934643592</v>
+        <v>0.52241986934649276</v>
       </c>
       <c r="J28" s="0">
-        <v>3.6120976169243022</v>
+        <v>3.612097616924359</v>
       </c>
       <c r="K28" s="0">
-        <v>-2.2512143002733183</v>
+        <v>-2.2512143002733467</v>
       </c>
       <c r="L28" s="0">
-        <v>2.766648465914844</v>
+        <v>2.7666484659147672</v>
       </c>
       <c r="M28" s="0"/>
       <c r="N28" s="0"/>
@@ -3189,31 +3801,31 @@
         <v>2030</v>
       </c>
       <c r="C29" s="0">
-        <v>166.76496394097842</v>
+        <v>166.76496394097839</v>
       </c>
       <c r="D29" s="0">
         <v>163.20348132848176</v>
       </c>
       <c r="E29" s="0">
-        <v>162.61272343277824</v>
+        <v>162.61272343277821</v>
       </c>
       <c r="F29" s="0">
         <v>1.709666665136524</v>
       </c>
       <c r="G29" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H29" s="0">
-        <v>3.5614826124966612</v>
+        <v>3.5614826124966328</v>
       </c>
       <c r="I29" s="0">
-        <v>0.59075789570351844</v>
+        <v>0.59075789570354686</v>
       </c>
       <c r="J29" s="0">
         <v>4.1522405082001796</v>
       </c>
       <c r="K29" s="0">
-        <v>-2.3872765672217611</v>
+        <v>-2.3872765672217895</v>
       </c>
       <c r="L29" s="0">
         <v>2.4286842534118227</v>
@@ -3236,31 +3848,31 @@
         <v>165.19379656327158</v>
       </c>
       <c r="D30" s="0">
-        <v>164.47896102783022</v>
+        <v>164.47896102783025</v>
       </c>
       <c r="E30" s="0">
-        <v>164.39026034623782</v>
+        <v>164.3902603462378</v>
       </c>
       <c r="F30" s="0">
-        <v>0.13849928742968132</v>
+        <v>0.13849928742970974</v>
       </c>
       <c r="G30" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H30" s="0">
-        <v>0.71483553544135248</v>
+        <v>0.71483553544132405</v>
       </c>
       <c r="I30" s="0">
-        <v>0.088700681592399633</v>
+        <v>0.088700681592456476</v>
       </c>
       <c r="J30" s="0">
-        <v>0.80353621703375211</v>
+        <v>0.80353621703378053</v>
       </c>
       <c r="K30" s="0">
-        <v>-0.6097396537621762</v>
+        <v>-0.60973965376220463</v>
       </c>
       <c r="L30" s="0">
-        <v>5.8017353875681312</v>
+        <v>5.8017353875671454</v>
       </c>
       <c r="M30" s="0"/>
       <c r="N30" s="0"/>
@@ -3273,34 +3885,34 @@
         <v>2025</v>
       </c>
       <c r="C31" s="0">
-        <v>165.21639502021844</v>
+        <v>165.21639502021847</v>
       </c>
       <c r="D31" s="0">
         <v>163.89090552699315</v>
       </c>
       <c r="E31" s="0">
-        <v>163.72499472037975</v>
+        <v>163.72499472037973</v>
       </c>
       <c r="F31" s="0">
-        <v>0.16109774437654778</v>
+        <v>0.16109774437660462</v>
       </c>
       <c r="G31" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H31" s="0">
-        <v>1.325489493225291</v>
+        <v>1.3254894932253194</v>
       </c>
       <c r="I31" s="0">
-        <v>0.16591080661339674</v>
+        <v>0.16591080661342517</v>
       </c>
       <c r="J31" s="0">
-        <v>1.4914002998386877</v>
+        <v>1.4914002998387446</v>
       </c>
       <c r="K31" s="0">
-        <v>-1.2750052796202453</v>
+        <v>-1.2750052796202738</v>
       </c>
       <c r="L31" s="0">
-        <v>9.25773545502107</v>
+        <v>9.2577354550181568</v>
       </c>
       <c r="M31" s="0"/>
       <c r="N31" s="0"/>
@@ -3316,22 +3928,22 @@
         <v>165.28897196681351</v>
       </c>
       <c r="D32" s="0">
-        <v>163.39477302566308</v>
+        <v>163.39477302566306</v>
       </c>
       <c r="E32" s="0">
         <v>163.16139254018776</v>
       </c>
       <c r="F32" s="0">
-        <v>0.2336746909716112</v>
+        <v>0.23367469097163962</v>
       </c>
       <c r="G32" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H32" s="0">
-        <v>1.894198941150421</v>
+        <v>1.8941989411504494</v>
       </c>
       <c r="I32" s="0">
-        <v>0.23338048547532253</v>
+        <v>0.23338048547529411</v>
       </c>
       <c r="J32" s="0">
         <v>2.1275794266257435</v>
@@ -3340,7 +3952,7 @@
         <v>-1.8386074598122377</v>
       </c>
       <c r="L32" s="0">
-        <v>9.1048774592547552</v>
+        <v>9.1048774592536486</v>
       </c>
       <c r="M32" s="0"/>
       <c r="N32" s="0"/>
@@ -3353,7 +3965,7 @@
         <v>2027</v>
       </c>
       <c r="C33" s="0">
-        <v>165.42417374238482</v>
+        <v>165.42417374238485</v>
       </c>
       <c r="D33" s="0">
         <v>162.99175619689834</v>
@@ -3362,25 +3974,25 @@
         <v>162.698715825823</v>
       </c>
       <c r="F33" s="0">
-        <v>0.36887646654292894</v>
+        <v>0.36887646654298578</v>
       </c>
       <c r="G33" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H33" s="0">
-        <v>2.4324175454864871</v>
+        <v>2.4324175454865156</v>
       </c>
       <c r="I33" s="0">
         <v>0.29304037107533532</v>
       </c>
       <c r="J33" s="0">
-        <v>2.7254579165618225</v>
+        <v>2.7254579165618509</v>
       </c>
       <c r="K33" s="0">
         <v>-2.3012841741769989</v>
       </c>
       <c r="L33" s="0">
-        <v>7.3885383421298858</v>
+        <v>7.3885383421288244</v>
       </c>
       <c r="M33" s="0"/>
       <c r="N33" s="0"/>
@@ -3393,34 +4005,34 @@
         <v>2028</v>
       </c>
       <c r="C34" s="0">
-        <v>165.6169906549494</v>
+        <v>165.61699065494943</v>
       </c>
       <c r="D34" s="0">
-        <v>162.66880106233475</v>
+        <v>162.66880106233478</v>
       </c>
       <c r="E34" s="0">
-        <v>162.32230473874097</v>
+        <v>162.32230473874094</v>
       </c>
       <c r="F34" s="0">
-        <v>0.56169337910750983</v>
+        <v>0.56169337910756667</v>
       </c>
       <c r="G34" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H34" s="0">
         <v>2.9481895926146535</v>
       </c>
       <c r="I34" s="0">
-        <v>0.34649632359378302</v>
+        <v>0.34649632359383986</v>
       </c>
       <c r="J34" s="0">
-        <v>3.2946859162084365</v>
+        <v>3.2946859162084934</v>
       </c>
       <c r="K34" s="0">
-        <v>-2.6776952612590321</v>
+        <v>-2.6776952612590605</v>
       </c>
       <c r="L34" s="0">
-        <v>5.8656306781530061</v>
+        <v>5.865630678152514</v>
       </c>
       <c r="M34" s="0"/>
       <c r="N34" s="0"/>
@@ -3433,34 +4045,34 @@
         <v>2029</v>
       </c>
       <c r="C35" s="0">
-        <v>165.86358790002362</v>
+        <v>165.86358790002359</v>
       </c>
       <c r="D35" s="0">
-        <v>162.41535206017431</v>
+        <v>162.41535206017434</v>
       </c>
       <c r="E35" s="0">
-        <v>162.02023833242629</v>
+        <v>162.02023833242632</v>
       </c>
       <c r="F35" s="0">
         <v>0.80829062418172271</v>
       </c>
       <c r="G35" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H35" s="0">
-        <v>3.4482358398493034</v>
+        <v>3.4482358398492465</v>
       </c>
       <c r="I35" s="0">
         <v>0.39511372774802567</v>
       </c>
       <c r="J35" s="0">
-        <v>3.843349567597329</v>
+        <v>3.8433495675972722</v>
       </c>
       <c r="K35" s="0">
-        <v>-2.9797616675737117</v>
+        <v>-2.9797616675736833</v>
       </c>
       <c r="L35" s="0">
-        <v>4.7549104896375169</v>
+        <v>4.7549104896374459</v>
       </c>
       <c r="M35" s="0"/>
       <c r="N35" s="0"/>
@@ -3476,22 +4088,22 @@
         <v>166.16095993962062</v>
       </c>
       <c r="D36" s="0">
-        <v>162.22283681275974</v>
+        <v>162.22283681275971</v>
       </c>
       <c r="E36" s="0">
         <v>161.78280304265581</v>
       </c>
       <c r="F36" s="0">
-        <v>1.1056626637787303</v>
+        <v>1.1056626637787588</v>
       </c>
       <c r="G36" s="0">
-        <v>0.055297275841894589</v>
+        <v>0.055297275841866167</v>
       </c>
       <c r="H36" s="0">
-        <v>3.9381231268608872</v>
+        <v>3.9381231268609156</v>
       </c>
       <c r="I36" s="0">
-        <v>0.44003377010392342</v>
+        <v>0.44003377010389499</v>
       </c>
       <c r="J36" s="0">
         <v>4.3781568969648106</v>
@@ -3500,7 +4112,7 @@
         <v>-3.2171969573441856</v>
       </c>
       <c r="L36" s="0">
-        <v>3.9597582883028282</v>
+        <v>3.9597582883027265</v>
       </c>
       <c r="M36" s="0">
         <v>173.25866293314667</v>
@@ -3518,13 +4130,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="18.85546875" customWidth="true"/>
-    <col min="3" max="3" width="14.28515625" customWidth="true"/>
-    <col min="4" max="4" width="14.28515625" customWidth="true"/>
-    <col min="5" max="5" width="18.85546875" customWidth="true"/>
-    <col min="6" max="6" width="14.28515625" customWidth="true"/>
-    <col min="7" max="7" width="17.140625" customWidth="true"/>
+    <col min="1" max="1" width="5.28515625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="12.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+    <col min="7" max="7" width="8.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3561,10 +4173,10 @@
         <v>162.59936305964357</v>
       </c>
       <c r="D2" s="0">
-        <v>162.14507925618148</v>
+        <v>162.1450792561815</v>
       </c>
       <c r="E2" s="0">
-        <v>0.45428380346208996</v>
+        <v>0.45428380346206154</v>
       </c>
       <c r="F2" s="0">
         <v>173.25866293314667</v>
@@ -3578,16 +4190,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="0">
-        <v>166.2391928015154</v>
+        <v>166.23919280151537</v>
       </c>
       <c r="C3" s="0">
         <v>162.77836104508094</v>
       </c>
       <c r="D3" s="0">
-        <v>162.20666765288877</v>
+        <v>162.20666765288874</v>
       </c>
       <c r="E3" s="0">
-        <v>0.57169339219217363</v>
+        <v>0.57169339219220205</v>
       </c>
       <c r="F3" s="0">
         <v>173.25866293314667</v>
@@ -3601,16 +4213,16 @@
         <v>7</v>
       </c>
       <c r="B4" s="0">
-        <v>166.54533035125223</v>
+        <v>166.54533035125226</v>
       </c>
       <c r="C4" s="0">
         <v>163.54829125244339</v>
       </c>
       <c r="D4" s="0">
-        <v>162.8247220283464</v>
+        <v>162.82472202834637</v>
       </c>
       <c r="E4" s="0">
-        <v>0.72356922409699109</v>
+        <v>0.72356922409701951</v>
       </c>
       <c r="F4" s="0">
         <v>173.25866293314667</v>
@@ -3624,16 +4236,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="0">
-        <v>166.76496394097842</v>
+        <v>166.76496394097839</v>
       </c>
       <c r="C5" s="0">
         <v>163.20348132848176</v>
       </c>
       <c r="D5" s="0">
-        <v>162.61272343277824</v>
+        <v>162.61272343277821</v>
       </c>
       <c r="E5" s="0">
-        <v>0.59075789570351844</v>
+        <v>0.59075789570354686</v>
       </c>
       <c r="F5" s="0">
         <v>173.25866293314667</v>
@@ -3650,13 +4262,13 @@
         <v>166.16095993962062</v>
       </c>
       <c r="C6" s="0">
-        <v>162.22283681275974</v>
+        <v>162.22283681275971</v>
       </c>
       <c r="D6" s="0">
         <v>161.78280304265581</v>
       </c>
       <c r="E6" s="0">
-        <v>0.44003377010392342</v>
+        <v>0.44003377010389499</v>
       </c>
       <c r="F6" s="0">
         <v>173.25866293314667</v>
@@ -3674,22 +4286,22 @@
   <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="15.42578125" customWidth="true"/>
-    <col min="3" max="3" width="15.42578125" customWidth="true"/>
-    <col min="4" max="4" width="15.42578125" customWidth="true"/>
-    <col min="5" max="5" width="15.42578125" customWidth="true"/>
-    <col min="6" max="6" width="15.42578125" customWidth="true"/>
-    <col min="7" max="7" width="15.42578125" customWidth="true"/>
-    <col min="8" max="8" width="15.42578125" customWidth="true"/>
-    <col min="9" max="9" width="15.42578125" customWidth="true"/>
-    <col min="10" max="10" width="15.42578125" customWidth="true"/>
-    <col min="11" max="11" width="15.42578125" customWidth="true"/>
-    <col min="12" max="12" width="15.42578125" customWidth="true"/>
-    <col min="13" max="13" width="15.42578125" customWidth="true"/>
-    <col min="14" max="14" width="15.42578125" customWidth="true"/>
-    <col min="15" max="15" width="15.42578125" customWidth="true"/>
-    <col min="16" max="16" width="15.42578125" customWidth="true"/>
+    <col min="1" max="1" width="5.140625" customWidth="true"/>
+    <col min="2" max="2" width="11.7109375" customWidth="true"/>
+    <col min="3" max="3" width="11.7109375" customWidth="true"/>
+    <col min="4" max="4" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="6" max="6" width="11.7109375" customWidth="true"/>
+    <col min="7" max="7" width="11.7109375" customWidth="true"/>
+    <col min="8" max="8" width="11.7109375" customWidth="true"/>
+    <col min="9" max="9" width="11.7109375" customWidth="true"/>
+    <col min="10" max="10" width="11.7109375" customWidth="true"/>
+    <col min="11" max="11" width="11.7109375" customWidth="true"/>
+    <col min="12" max="12" width="11.7109375" customWidth="true"/>
+    <col min="13" max="13" width="11.7109375" customWidth="true"/>
+    <col min="14" max="14" width="11.7109375" customWidth="true"/>
+    <col min="15" max="15" width="11.7109375" customWidth="true"/>
+    <col min="16" max="16" width="11.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3806,7 +4418,7 @@
         <v>164.38619132866143</v>
       </c>
       <c r="E3" s="0">
-        <v>165.17908275339119</v>
+        <v>165.17908275339116</v>
       </c>
       <c r="F3" s="0">
         <v>164.56953805219825</v>
@@ -3818,28 +4430,28 @@
         <v>165.17701487907493</v>
       </c>
       <c r="I3" s="0">
-        <v>164.67302725600655</v>
+        <v>164.67302725600658</v>
       </c>
       <c r="J3" s="0">
-        <v>164.54470676967651</v>
+        <v>164.54470676967648</v>
       </c>
       <c r="K3" s="0">
-        <v>165.18959527748223</v>
+        <v>165.1895952774822</v>
       </c>
       <c r="L3" s="0">
-        <v>164.57953360994259</v>
+        <v>164.57953360994256</v>
       </c>
       <c r="M3" s="0">
-        <v>164.47111208956096</v>
+        <v>164.47111208956099</v>
       </c>
       <c r="N3" s="0">
         <v>165.19379656327158</v>
       </c>
       <c r="O3" s="0">
-        <v>164.47896102783022</v>
+        <v>164.47896102783025</v>
       </c>
       <c r="P3" s="0">
-        <v>164.39026034623782</v>
+        <v>164.3902603462378</v>
       </c>
     </row>
     <row r="4">
@@ -3847,13 +4459,13 @@
         <v>2025</v>
       </c>
       <c r="B4" s="0">
-        <v>165.30180939577485</v>
+        <v>165.30180939577482</v>
       </c>
       <c r="C4" s="0">
         <v>163.97336291396618</v>
       </c>
       <c r="D4" s="0">
-        <v>163.80656719074852</v>
+        <v>163.8065671907485</v>
       </c>
       <c r="E4" s="0">
         <v>165.2711738744573</v>
@@ -3862,34 +4474,34 @@
         <v>164.13567579262497</v>
       </c>
       <c r="G4" s="0">
-        <v>163.93019403217454</v>
+        <v>163.93019403217457</v>
       </c>
       <c r="H4" s="0">
-        <v>165.35738468088493</v>
+        <v>165.35738468088491</v>
       </c>
       <c r="I4" s="0">
         <v>164.41462707096798</v>
       </c>
       <c r="J4" s="0">
-        <v>164.16796436844356</v>
+        <v>164.16796436844359</v>
       </c>
       <c r="K4" s="0">
         <v>165.31187985390261</v>
       </c>
       <c r="L4" s="0">
-        <v>164.17326296256704</v>
+        <v>164.17326296256701</v>
       </c>
       <c r="M4" s="0">
         <v>163.96729971165348</v>
       </c>
       <c r="N4" s="0">
-        <v>165.21639502021844</v>
+        <v>165.21639502021847</v>
       </c>
       <c r="O4" s="0">
         <v>163.89090552699315</v>
       </c>
       <c r="P4" s="0">
-        <v>163.72499472037975</v>
+        <v>163.72499472037973</v>
       </c>
     </row>
     <row r="5">
@@ -3903,40 +4515,40 @@
         <v>163.55132054552689</v>
       </c>
       <c r="D5" s="0">
-        <v>163.31537043441051</v>
+        <v>163.31537043441048</v>
       </c>
       <c r="E5" s="0">
-        <v>165.39175668478583</v>
+        <v>165.39175668478586</v>
       </c>
       <c r="F5" s="0">
-        <v>163.75690974914642</v>
+        <v>163.75690974914644</v>
       </c>
       <c r="G5" s="0">
-        <v>163.46416615192811</v>
+        <v>163.46416615192814</v>
       </c>
       <c r="H5" s="0">
-        <v>165.55205244119804</v>
+        <v>165.55205244119807</v>
       </c>
       <c r="I5" s="0">
-        <v>164.18191529280375</v>
+        <v>164.18191529280378</v>
       </c>
       <c r="J5" s="0">
-        <v>163.82594933505652</v>
+        <v>163.82594933505655</v>
       </c>
       <c r="K5" s="0">
-        <v>165.48313209048638</v>
+        <v>165.48313209048629</v>
       </c>
       <c r="L5" s="0">
-        <v>163.83883059982793</v>
+        <v>163.8388305998279</v>
       </c>
       <c r="M5" s="0">
-        <v>163.54448971731847</v>
+        <v>163.54448971731844</v>
       </c>
       <c r="N5" s="0">
         <v>165.28897196681351</v>
       </c>
       <c r="O5" s="0">
-        <v>163.39477302566308</v>
+        <v>163.39477302566306</v>
       </c>
       <c r="P5" s="0">
         <v>163.16139254018776</v>
@@ -3950,40 +4562,40 @@
         <v>165.66473162170803</v>
       </c>
       <c r="C6" s="0">
-        <v>163.21259564728871</v>
+        <v>163.21259564728874</v>
       </c>
       <c r="D6" s="0">
-        <v>162.91468122506888</v>
+        <v>162.91468122506885</v>
       </c>
       <c r="E6" s="0">
-        <v>165.55366021191776</v>
+        <v>165.55366021191779</v>
       </c>
       <c r="F6" s="0">
-        <v>163.43991055875335</v>
+        <v>163.43991055875333</v>
       </c>
       <c r="G6" s="0">
-        <v>163.06813799635404</v>
+        <v>163.06813799635407</v>
       </c>
       <c r="H6" s="0">
-        <v>165.77368046029869</v>
+        <v>165.77368046029872</v>
       </c>
       <c r="I6" s="0">
-        <v>163.98491070706655</v>
+        <v>163.98491070706658</v>
       </c>
       <c r="J6" s="0">
-        <v>163.52743712330891</v>
+        <v>163.52743712330894</v>
       </c>
       <c r="K6" s="0">
         <v>165.71745574966292</v>
       </c>
       <c r="L6" s="0">
-        <v>163.58262820418611</v>
+        <v>163.58262820418608</v>
       </c>
       <c r="M6" s="0">
-        <v>163.20712392957535</v>
+        <v>163.20712392957537</v>
       </c>
       <c r="N6" s="0">
-        <v>165.42417374238482</v>
+        <v>165.42417374238485</v>
       </c>
       <c r="O6" s="0">
         <v>162.99175619689834</v>
@@ -3997,49 +4609,49 @@
         <v>2028</v>
       </c>
       <c r="B7" s="0">
-        <v>165.92452240193279</v>
+        <v>165.92452240193282</v>
       </c>
       <c r="C7" s="0">
-        <v>162.94645336639951</v>
+        <v>162.94645336639954</v>
       </c>
       <c r="D7" s="0">
-        <v>162.59229900031778</v>
+        <v>162.59229900031775</v>
       </c>
       <c r="E7" s="0">
-        <v>165.75165500037542</v>
+        <v>165.75165500037545</v>
       </c>
       <c r="F7" s="0">
-        <v>163.17580300969121</v>
+        <v>163.17580300969129</v>
       </c>
       <c r="G7" s="0">
-        <v>162.73191661247608</v>
+        <v>162.73191661247611</v>
       </c>
       <c r="H7" s="0">
-        <v>166.01647565182861</v>
+        <v>166.01647565182864</v>
       </c>
       <c r="I7" s="0">
-        <v>163.81713336301107</v>
+        <v>163.81713336301104</v>
       </c>
       <c r="J7" s="0">
-        <v>163.2650296628193</v>
+        <v>163.26502966281927</v>
       </c>
       <c r="K7" s="0">
-        <v>166.01099013827525</v>
+        <v>166.01099013827528</v>
       </c>
       <c r="L7" s="0">
-        <v>163.39575223633108</v>
+        <v>163.39575223633111</v>
       </c>
       <c r="M7" s="0">
         <v>162.9446861805086</v>
       </c>
       <c r="N7" s="0">
-        <v>165.6169906549494</v>
+        <v>165.61699065494943</v>
       </c>
       <c r="O7" s="0">
-        <v>162.66880106233475</v>
+        <v>162.66880106233478</v>
       </c>
       <c r="P7" s="0">
-        <v>162.32230473874097</v>
+        <v>162.32230473874094</v>
       </c>
     </row>
     <row r="8">
@@ -4047,49 +4659,49 @@
         <v>2029</v>
       </c>
       <c r="B8" s="0">
-        <v>166.23235054936822</v>
+        <v>166.23235054936825</v>
       </c>
       <c r="C8" s="0">
-        <v>162.74433075594322</v>
+        <v>162.74433075594325</v>
       </c>
       <c r="D8" s="0">
-        <v>162.33840659579766</v>
+        <v>162.33840659579769</v>
       </c>
       <c r="E8" s="0">
-        <v>165.98140207954998</v>
+        <v>165.98140207955001</v>
       </c>
       <c r="F8" s="0">
-        <v>162.95730873361413</v>
+        <v>162.9573087336141</v>
       </c>
       <c r="G8" s="0">
-        <v>162.44709821255765</v>
+        <v>162.44709821255762</v>
       </c>
       <c r="H8" s="0">
         <v>166.2752704578138</v>
       </c>
       <c r="I8" s="0">
-        <v>163.67315319301497</v>
+        <v>163.673153193015</v>
       </c>
       <c r="J8" s="0">
-        <v>163.03254975774746</v>
+        <v>163.03254975774743</v>
       </c>
       <c r="K8" s="0">
-        <v>166.36088331665098</v>
+        <v>166.36088331665101</v>
       </c>
       <c r="L8" s="0">
-        <v>163.27120556907312</v>
+        <v>163.27120556907315</v>
       </c>
       <c r="M8" s="0">
-        <v>162.74878569972668</v>
+        <v>162.74878569972665</v>
       </c>
       <c r="N8" s="0">
-        <v>165.86358790002362</v>
+        <v>165.86358790002359</v>
       </c>
       <c r="O8" s="0">
-        <v>162.41535206017431</v>
+        <v>162.41535206017434</v>
       </c>
       <c r="P8" s="0">
-        <v>162.02023833242629</v>
+        <v>162.02023833242632</v>
       </c>
     </row>
     <row r="9">
@@ -4103,40 +4715,40 @@
         <v>162.59936305964357</v>
       </c>
       <c r="D9" s="0">
-        <v>162.14507925618148</v>
+        <v>162.1450792561815</v>
       </c>
       <c r="E9" s="0">
-        <v>166.2391928015154</v>
+        <v>166.23919280151537</v>
       </c>
       <c r="F9" s="0">
         <v>162.77836104508094</v>
       </c>
       <c r="G9" s="0">
-        <v>162.20666765288877</v>
+        <v>162.20666765288874</v>
       </c>
       <c r="H9" s="0">
-        <v>166.54533035125223</v>
+        <v>166.54533035125226</v>
       </c>
       <c r="I9" s="0">
         <v>163.54829125244339</v>
       </c>
       <c r="J9" s="0">
-        <v>162.8247220283464</v>
+        <v>162.82472202834637</v>
       </c>
       <c r="K9" s="0">
-        <v>166.76496394097842</v>
+        <v>166.76496394097839</v>
       </c>
       <c r="L9" s="0">
         <v>163.20348132848176</v>
       </c>
       <c r="M9" s="0">
-        <v>162.61272343277824</v>
+        <v>162.61272343277821</v>
       </c>
       <c r="N9" s="0">
         <v>166.16095993962062</v>
       </c>
       <c r="O9" s="0">
-        <v>162.22283681275974</v>
+        <v>162.22283681275971</v>
       </c>
       <c r="P9" s="0">
         <v>161.78280304265581</v>
@@ -4151,17 +4763,17 @@
   <dimension ref="A1:K106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="true"/>
-    <col min="2" max="2" width="10.28515625" customWidth="true"/>
-    <col min="3" max="3" width="5.7109375" customWidth="true"/>
-    <col min="4" max="4" width="27.28515625" customWidth="true"/>
-    <col min="5" max="5" width="23.140625" customWidth="true"/>
-    <col min="6" max="6" width="29" customWidth="true"/>
-    <col min="7" max="7" width="31.7109375" customWidth="true"/>
+    <col min="1" max="1" width="5.28515625" customWidth="true"/>
+    <col min="2" max="2" width="5.7109375" customWidth="true"/>
+    <col min="3" max="3" width="5.140625" customWidth="true"/>
+    <col min="4" max="4" width="13.7109375" customWidth="true"/>
+    <col min="5" max="5" width="12.7109375" customWidth="true"/>
+    <col min="6" max="6" width="16.7109375" customWidth="true"/>
+    <col min="7" max="7" width="18.7109375" customWidth="true"/>
     <col min="8" max="8" width="11.7109375" customWidth="true"/>
     <col min="9" max="9" width="11.7109375" customWidth="true"/>
-    <col min="10" max="10" width="17.140625" customWidth="true"/>
-    <col min="11" max="11" width="17.140625" customWidth="true"/>
+    <col min="10" max="10" width="11.7109375" customWidth="true"/>
+    <col min="11" max="11" width="12.7109375" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4534,13 +5146,13 @@
         <v>11273.548854276332</v>
       </c>
       <c r="G11" s="0">
-        <v>4.8950400129231344</v>
+        <v>4.8950400129231326</v>
       </c>
       <c r="H11" s="0">
         <v>272.34264069655768</v>
       </c>
       <c r="I11" s="0">
-        <v>5.518447272932641</v>
+        <v>5.5184472729326384</v>
       </c>
       <c r="J11" s="0">
         <v>4964.8499786519487</v>
@@ -4569,13 +5181,13 @@
         <v>11562.983320709014</v>
       </c>
       <c r="G12" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H12" s="0">
         <v>270.34804295124519</v>
       </c>
       <c r="I12" s="0">
-        <v>5.0481067536983755</v>
+        <v>5.0481067536983746</v>
       </c>
       <c r="J12" s="0">
         <v>4962.7729246100753</v>
@@ -4604,13 +5216,13 @@
         <v>11848.119367481104</v>
       </c>
       <c r="G13" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H13" s="0">
         <v>268.35440264276286</v>
       </c>
       <c r="I13" s="0">
-        <v>4.6132866153768681</v>
+        <v>4.6132866153768655</v>
       </c>
       <c r="J13" s="0">
         <v>4958.3727264234776</v>
@@ -4639,13 +5251,13 @@
         <v>12128.307560666564</v>
       </c>
       <c r="G14" s="0">
-        <v>3.4726690910316687</v>
+        <v>3.4726690910316678</v>
       </c>
       <c r="H14" s="0">
         <v>266.36239886547594</v>
       </c>
       <c r="I14" s="0">
-        <v>4.2117598792452471</v>
+        <v>4.2117598792452462</v>
       </c>
       <c r="J14" s="0">
         <v>4951.8377986488385</v>
@@ -4674,13 +5286,13 @@
         <v>12403.213235664984</v>
       </c>
       <c r="G15" s="0">
-        <v>3.0971752971880306</v>
+        <v>3.0971752971880293</v>
       </c>
       <c r="H15" s="0">
         <v>264.37267868637747</v>
       </c>
       <c r="I15" s="0">
-        <v>3.8414925639257214</v>
+        <v>3.8414925639257191</v>
       </c>
       <c r="J15" s="0">
         <v>4943.3305587725963</v>
@@ -4779,13 +5391,13 @@
         <v>11273.548854276332</v>
       </c>
       <c r="G18" s="0">
-        <v>4.8950400129231344</v>
+        <v>4.8950400129231326</v>
       </c>
       <c r="H18" s="0">
         <v>267.05399032181731</v>
       </c>
       <c r="I18" s="0">
-        <v>5.518447272932641</v>
+        <v>5.5184472729326384</v>
       </c>
       <c r="J18" s="0">
         <v>4964.8499786519487</v>
@@ -4814,13 +5426,13 @@
         <v>11562.983320709014</v>
       </c>
       <c r="G19" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H19" s="0">
         <v>263.49059878611888</v>
       </c>
       <c r="I19" s="0">
-        <v>5.0481067536983755</v>
+        <v>5.0481067536983746</v>
       </c>
       <c r="J19" s="0">
         <v>4962.7729246100753</v>
@@ -4849,13 +5461,13 @@
         <v>11848.119367481104</v>
       </c>
       <c r="G20" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H20" s="0">
         <v>260.01771460336039</v>
       </c>
       <c r="I20" s="0">
-        <v>4.6132866153768681</v>
+        <v>4.6132866153768655</v>
       </c>
       <c r="J20" s="0">
         <v>4958.3727264234776</v>
@@ -4884,13 +5496,13 @@
         <v>12128.307560666564</v>
       </c>
       <c r="G21" s="0">
-        <v>3.4726690910316687</v>
+        <v>3.4726690910316678</v>
       </c>
       <c r="H21" s="0">
         <v>256.63187574149555</v>
       </c>
       <c r="I21" s="0">
-        <v>4.2117598792452471</v>
+        <v>4.2117598792452462</v>
       </c>
       <c r="J21" s="0">
         <v>4951.8377986488385</v>
@@ -4919,13 +5531,13 @@
         <v>12403.213235664984</v>
       </c>
       <c r="G22" s="0">
-        <v>3.0971752971880306</v>
+        <v>3.0971752971880293</v>
       </c>
       <c r="H22" s="0">
         <v>253.32980394562759</v>
       </c>
       <c r="I22" s="0">
-        <v>3.8414925639257214</v>
+        <v>3.8414925639257191</v>
       </c>
       <c r="J22" s="0">
         <v>4943.3305587725963</v>
@@ -5234,13 +5846,13 @@
         <v>10951.715306495595</v>
       </c>
       <c r="G31" s="0">
-        <v>5.7019017889405408</v>
+        <v>5.7019017889405399</v>
       </c>
       <c r="H31" s="0">
         <v>275.22524610906447</v>
       </c>
       <c r="I31" s="0">
-        <v>6.2445605098074735</v>
+        <v>6.2445605098074726</v>
       </c>
       <c r="J31" s="0">
         <v>4965.3421191658026</v>
@@ -5269,13 +5881,13 @@
         <v>11228.830076099021</v>
       </c>
       <c r="G32" s="0">
-        <v>5.1832845781137689</v>
+        <v>5.183284578113768</v>
       </c>
       <c r="H32" s="0">
         <v>273.66052511000248</v>
       </c>
       <c r="I32" s="0">
-        <v>5.8202221763704109</v>
+        <v>5.8202221763704101</v>
       </c>
       <c r="J32" s="0">
         <v>4967.0775544139915</v>
@@ -5304,13 +5916,13 @@
         <v>11502.357593500228</v>
       </c>
       <c r="G33" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H33" s="0">
         <v>272.08719371663386</v>
       </c>
       <c r="I33" s="0">
-        <v>5.4197248617133846</v>
+        <v>5.4197248617133837</v>
       </c>
       <c r="J33" s="0">
         <v>4966.8360737222874</v>
@@ -5339,13 +5951,13 @@
         <v>11771.285389167622</v>
       </c>
       <c r="G34" s="0">
-        <v>4.2832724070340307</v>
+        <v>4.2832724070340298</v>
       </c>
       <c r="H34" s="0">
         <v>270.50619166419477</v>
       </c>
       <c r="I34" s="0">
-        <v>5.041962190274452</v>
+        <v>5.0419621902744503</v>
       </c>
       <c r="J34" s="0">
         <v>4964.8755355182457</v>
@@ -5374,13 +5986,13 @@
         <v>12035.083991282194</v>
       </c>
       <c r="G35" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H35" s="0">
         <v>268.91841757737831</v>
       </c>
       <c r="I35" s="0">
-        <v>4.6860847844177584</v>
+        <v>4.6860847844177567</v>
       </c>
       <c r="J35" s="0">
         <v>4961.421981860155</v>
@@ -5409,13 +6021,13 @@
         <v>12293.535718208348</v>
       </c>
       <c r="G36" s="0">
-        <v>3.5395360290126079</v>
+        <v>3.5395360290126066</v>
       </c>
       <c r="H36" s="0">
         <v>267.32473023027075</v>
       </c>
       <c r="I36" s="0">
-        <v>4.3513412598551833</v>
+        <v>4.3513412598551815</v>
       </c>
       <c r="J36" s="0">
         <v>4956.675361145908</v>
@@ -5479,13 +6091,13 @@
         <v>10951.715306495595</v>
       </c>
       <c r="G38" s="0">
-        <v>5.7019017889405408</v>
+        <v>5.7019017889405399</v>
       </c>
       <c r="H38" s="0">
         <v>270.79874250945323</v>
       </c>
       <c r="I38" s="0">
-        <v>6.2445605098074735</v>
+        <v>6.2445605098074726</v>
       </c>
       <c r="J38" s="0">
         <v>4965.3421191658026</v>
@@ -5514,13 +6126,13 @@
         <v>11228.830076099021</v>
       </c>
       <c r="G39" s="0">
-        <v>5.1832845781137689</v>
+        <v>5.183284578113768</v>
       </c>
       <c r="H39" s="0">
         <v>267.17800096714444</v>
       </c>
       <c r="I39" s="0">
-        <v>5.8202221763704109</v>
+        <v>5.8202221763704101</v>
       </c>
       <c r="J39" s="0">
         <v>4967.0775544139915</v>
@@ -5549,13 +6161,13 @@
         <v>11502.357593500228</v>
       </c>
       <c r="G40" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H40" s="0">
         <v>263.64739184618224</v>
       </c>
       <c r="I40" s="0">
-        <v>5.4197248617133846</v>
+        <v>5.4197248617133837</v>
       </c>
       <c r="J40" s="0">
         <v>4966.8360737222874</v>
@@ -5584,13 +6196,13 @@
         <v>11771.285389167622</v>
       </c>
       <c r="G41" s="0">
-        <v>4.2832724070340307</v>
+        <v>4.2832724070340298</v>
       </c>
       <c r="H41" s="0">
         <v>260.20358558167902</v>
       </c>
       <c r="I41" s="0">
-        <v>5.041962190274452</v>
+        <v>5.0419621902744503</v>
       </c>
       <c r="J41" s="0">
         <v>4964.8755355182457</v>
@@ -5619,13 +6231,13 @@
         <v>12035.083991282194</v>
       </c>
       <c r="G42" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H42" s="0">
         <v>256.84342539793977</v>
       </c>
       <c r="I42" s="0">
-        <v>4.6860847844177584</v>
+        <v>4.6860847844177567</v>
       </c>
       <c r="J42" s="0">
         <v>4961.421981860155</v>
@@ -5654,13 +6266,13 @@
         <v>12293.535718208348</v>
       </c>
       <c r="G43" s="0">
-        <v>3.5395360290126079</v>
+        <v>3.5395360290126066</v>
       </c>
       <c r="H43" s="0">
         <v>253.56391534929423</v>
       </c>
       <c r="I43" s="0">
-        <v>4.3513412598551833</v>
+        <v>4.3513412598551815</v>
       </c>
       <c r="J43" s="0">
         <v>4956.675361145908</v>
@@ -6039,13 +6651,13 @@
         <v>11463.725653073918</v>
       </c>
       <c r="G54" s="0">
-        <v>5.0853648605063242</v>
+        <v>5.0853648605063224</v>
       </c>
       <c r="H54" s="0">
         <v>273.83482532475165</v>
       </c>
       <c r="I54" s="0">
-        <v>5.8297227606627011</v>
+        <v>5.8297227606626993</v>
       </c>
       <c r="J54" s="0">
         <v>4956.3381108871517</v>
@@ -6074,13 +6686,13 @@
         <v>11716.088136896597</v>
       </c>
       <c r="G55" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H55" s="0">
         <v>272.67118985015077</v>
       </c>
       <c r="I55" s="0">
-        <v>5.520431236935746</v>
+        <v>5.5204312369357451</v>
       </c>
       <c r="J55" s="0">
         <v>4952.1629005952391</v>
@@ -6109,13 +6721,13 @@
         <v>11960.43229598056</v>
       </c>
       <c r="G56" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H56" s="0">
         <v>271.49339508509757</v>
       </c>
       <c r="I56" s="0">
-        <v>5.2216229476312543</v>
+        <v>5.2216229476312535</v>
       </c>
       <c r="J56" s="0">
         <v>4947.1718281996455</v>
@@ -6144,13 +6756,13 @@
         <v>12196.515676800944</v>
       </c>
       <c r="G57" s="0">
-        <v>4.0450778850176734</v>
+        <v>4.0450778850176716</v>
       </c>
       <c r="H57" s="0">
         <v>270.30249952925908</v>
       </c>
       <c r="I57" s="0">
-        <v>4.9335855838498857</v>
+        <v>4.9335855838498839</v>
       </c>
       <c r="J57" s="0">
         <v>4941.5845485528753</v>
@@ -6284,13 +6896,13 @@
         <v>11463.725653073918</v>
       </c>
       <c r="G61" s="0">
-        <v>5.0853648605063242</v>
+        <v>5.0853648605063224</v>
       </c>
       <c r="H61" s="0">
         <v>263.80167026954791</v>
       </c>
       <c r="I61" s="0">
-        <v>5.8297227606627011</v>
+        <v>5.8297227606626993</v>
       </c>
       <c r="J61" s="0">
         <v>4956.3381108871517</v>
@@ -6319,13 +6931,13 @@
         <v>11716.088136896597</v>
       </c>
       <c r="G62" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H62" s="0">
         <v>260.38572680394134</v>
       </c>
       <c r="I62" s="0">
-        <v>5.520431236935746</v>
+        <v>5.5204312369357451</v>
       </c>
       <c r="J62" s="0">
         <v>4952.1629005952391</v>
@@ -6354,13 +6966,13 @@
         <v>11960.43229598056</v>
       </c>
       <c r="G63" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H63" s="0">
         <v>257.04987689443396</v>
       </c>
       <c r="I63" s="0">
-        <v>5.2216229476312543</v>
+        <v>5.2216229476312535</v>
       </c>
       <c r="J63" s="0">
         <v>4947.1718281996455</v>
@@ -6389,13 +7001,13 @@
         <v>12196.515676800944</v>
       </c>
       <c r="G64" s="0">
-        <v>4.0450778850176734</v>
+        <v>4.0450778850176716</v>
       </c>
       <c r="H64" s="0">
         <v>253.79144009922103</v>
       </c>
       <c r="I64" s="0">
-        <v>4.9335855838498857</v>
+        <v>4.9335855838498839</v>
       </c>
       <c r="J64" s="0">
         <v>4941.5845485528753</v>
@@ -6774,13 +7386,13 @@
         <v>11517.178324585864</v>
       </c>
       <c r="G75" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H75" s="0">
         <v>272.08719371663386</v>
       </c>
       <c r="I75" s="0">
-        <v>5.426708150494024</v>
+        <v>5.4267081504940231</v>
       </c>
       <c r="J75" s="0">
         <v>4959.7216252327062</v>
@@ -6809,13 +7421,13 @@
         <v>11790.582474086703</v>
       </c>
       <c r="G76" s="0">
-        <v>4.2832724070340307</v>
+        <v>4.2832724070340298</v>
       </c>
       <c r="H76" s="0">
         <v>270.50619166419477</v>
       </c>
       <c r="I76" s="0">
-        <v>5.0502276574114608</v>
+        <v>5.05022765741146</v>
       </c>
       <c r="J76" s="0">
         <v>4953.6510108132097</v>
@@ -6844,13 +7456,13 @@
         <v>12059.067313921241</v>
       </c>
       <c r="G77" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H77" s="0">
         <v>268.91841757737831</v>
       </c>
       <c r="I77" s="0">
-        <v>4.6954231391297023</v>
+        <v>4.6954231391296997</v>
       </c>
       <c r="J77" s="0">
         <v>4945.1188672135368</v>
@@ -6879,13 +7491,13 @@
         <v>12322.361028364183</v>
       </c>
       <c r="G78" s="0">
-        <v>3.5395360290126074</v>
+        <v>3.5395360290126066</v>
       </c>
       <c r="H78" s="0">
         <v>267.32473023027075</v>
       </c>
       <c r="I78" s="0">
-        <v>4.361544082239587</v>
+        <v>4.3615440822395861</v>
       </c>
       <c r="J78" s="0">
         <v>4934.3089491566398</v>
@@ -7019,13 +7631,13 @@
         <v>11517.178324585864</v>
       </c>
       <c r="G82" s="0">
-        <v>4.7118382624236723</v>
+        <v>4.7118382624236714</v>
       </c>
       <c r="H82" s="0">
         <v>263.64739184618224</v>
       </c>
       <c r="I82" s="0">
-        <v>5.426708150494024</v>
+        <v>5.4267081504940231</v>
       </c>
       <c r="J82" s="0">
         <v>4959.7216252327062</v>
@@ -7054,13 +7666,13 @@
         <v>11790.582474086703</v>
       </c>
       <c r="G83" s="0">
-        <v>4.2832724070340307</v>
+        <v>4.2832724070340298</v>
       </c>
       <c r="H83" s="0">
         <v>260.20358558167902</v>
       </c>
       <c r="I83" s="0">
-        <v>5.0502276574114608</v>
+        <v>5.05022765741146</v>
       </c>
       <c r="J83" s="0">
         <v>4953.6510108132097</v>
@@ -7089,13 +7701,13 @@
         <v>12059.067313921241</v>
       </c>
       <c r="G84" s="0">
-        <v>3.8936868141611636</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H84" s="0">
         <v>256.84342539793977</v>
       </c>
       <c r="I84" s="0">
-        <v>4.6954231391297023</v>
+        <v>4.6954231391296997</v>
       </c>
       <c r="J84" s="0">
         <v>4945.1188672135368</v>
@@ -7124,13 +7736,13 @@
         <v>12322.361028364183</v>
       </c>
       <c r="G85" s="0">
-        <v>3.5395360290126074</v>
+        <v>3.5395360290126066</v>
       </c>
       <c r="H85" s="0">
         <v>253.56391534929423</v>
       </c>
       <c r="I85" s="0">
-        <v>4.361544082239587</v>
+        <v>4.3615440822395861</v>
       </c>
       <c r="J85" s="0">
         <v>4934.3089491566398</v>
@@ -7404,13 +8016,13 @@
         <v>10683.037544206034</v>
       </c>
       <c r="G93" s="0">
-        <v>6.1539147527150693</v>
+        <v>6.1539147527150675</v>
       </c>
       <c r="H93" s="0">
         <v>276.33182562206338</v>
       </c>
       <c r="I93" s="0">
-        <v>6.5742502347098473</v>
+        <v>6.5742502347098464</v>
       </c>
       <c r="J93" s="0">
         <v>4961.6731820418327</v>
@@ -7474,13 +8086,13 @@
         <v>11327.377261222491</v>
       </c>
       <c r="G95" s="0">
-        <v>4.8950400129231344</v>
+        <v>4.8950400129231326</v>
       </c>
       <c r="H95" s="0">
         <v>272.34264069655768</v>
       </c>
       <c r="I95" s="0">
-        <v>5.5447964935159764</v>
+        <v>5.5447964935159737</v>
       </c>
       <c r="J95" s="0">
         <v>4973.763387631232</v>
@@ -7509,13 +8121,13 @@
         <v>11642.784702480307</v>
       </c>
       <c r="G96" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H96" s="0">
         <v>270.34804295124519</v>
       </c>
       <c r="I96" s="0">
-        <v>5.0829460233834434</v>
+        <v>5.0829460233834425</v>
       </c>
       <c r="J96" s="0">
         <v>4975.5778847342535</v>
@@ -7544,13 +8156,13 @@
         <v>11957.906477264474</v>
       </c>
       <c r="G97" s="0">
-        <v>3.8936868141611631</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H97" s="0">
         <v>268.35440264276286</v>
       </c>
       <c r="I97" s="0">
-        <v>4.656034277549705</v>
+        <v>4.6560342775497032</v>
       </c>
       <c r="J97" s="0">
         <v>4974.7691248761766</v>
@@ -7579,13 +8191,13 @@
         <v>12272.08041548608</v>
       </c>
       <c r="G98" s="0">
-        <v>3.4726690910316682</v>
+        <v>3.4726690910316673</v>
       </c>
       <c r="H98" s="0">
         <v>266.36239886547594</v>
       </c>
       <c r="I98" s="0">
-        <v>4.2616874341513586</v>
+        <v>4.2616874341513569</v>
       </c>
       <c r="J98" s="0">
         <v>4971.565905127808</v>
@@ -7614,13 +8226,13 @@
         <v>12584.953004072098</v>
       </c>
       <c r="G99" s="0">
-        <v>3.0971752971880306</v>
+        <v>3.0971752971880289</v>
       </c>
       <c r="H99" s="0">
         <v>264.37267868637747</v>
       </c>
       <c r="I99" s="0">
-        <v>3.8977805560484398</v>
+        <v>3.8977805560484375</v>
       </c>
       <c r="J99" s="0">
         <v>4966.1714963135119</v>
@@ -7649,13 +8261,13 @@
         <v>10683.037544206034</v>
       </c>
       <c r="G100" s="0">
-        <v>6.1539147527150693</v>
+        <v>6.1539147527150675</v>
       </c>
       <c r="H100" s="0">
         <v>274.46714652888301</v>
       </c>
       <c r="I100" s="0">
-        <v>6.5742502347098473</v>
+        <v>6.5742502347098464</v>
       </c>
       <c r="J100" s="0">
         <v>4961.6731820418327</v>
@@ -7719,13 +8331,13 @@
         <v>11327.377261222491</v>
       </c>
       <c r="G102" s="0">
-        <v>4.8950400129231344</v>
+        <v>4.8950400129231326</v>
       </c>
       <c r="H102" s="0">
         <v>267.05399032181731</v>
       </c>
       <c r="I102" s="0">
-        <v>5.5447964935159764</v>
+        <v>5.5447964935159737</v>
       </c>
       <c r="J102" s="0">
         <v>4973.763387631232</v>
@@ -7754,13 +8366,13 @@
         <v>11642.784702480307</v>
       </c>
       <c r="G103" s="0">
-        <v>4.3657476740084391</v>
+        <v>4.3657476740084382</v>
       </c>
       <c r="H103" s="0">
         <v>263.49059878611888</v>
       </c>
       <c r="I103" s="0">
-        <v>5.0829460233834434</v>
+        <v>5.0829460233834425</v>
       </c>
       <c r="J103" s="0">
         <v>4975.5778847342535</v>
@@ -7789,13 +8401,13 @@
         <v>11957.906477264474</v>
       </c>
       <c r="G104" s="0">
-        <v>3.8936868141611631</v>
+        <v>3.8936868141611618</v>
       </c>
       <c r="H104" s="0">
         <v>260.01771460336039</v>
       </c>
       <c r="I104" s="0">
-        <v>4.656034277549705</v>
+        <v>4.6560342775497032</v>
       </c>
       <c r="J104" s="0">
         <v>4974.7691248761766</v>
@@ -7824,13 +8436,13 @@
         <v>12272.08041548608</v>
       </c>
       <c r="G105" s="0">
-        <v>3.4726690910316682</v>
+        <v>3.4726690910316673</v>
       </c>
       <c r="H105" s="0">
         <v>256.63187574149555</v>
       </c>
       <c r="I105" s="0">
-        <v>4.2616874341513586</v>
+        <v>4.2616874341513569</v>
       </c>
       <c r="J105" s="0">
         <v>4971.565905127808</v>
@@ -7859,13 +8471,13 @@
         <v>12584.953004072098</v>
       </c>
       <c r="G106" s="0">
-        <v>3.0971752971880306</v>
+        <v>3.0971752971880289</v>
       </c>
       <c r="H106" s="0">
         <v>253.32980394562759</v>
       </c>
       <c r="I106" s="0">
-        <v>3.8977805560484398</v>
+        <v>3.8977805560484375</v>
       </c>
       <c r="J106" s="0">
         <v>4966.1714963135119</v>

</xml_diff>